<commit_message>
Implemented food waste calculations
</commit_message>
<xml_diff>
--- a/data/prod_parameters/Diet.xlsx
+++ b/data/prod_parameters/Diet.xlsx
@@ -4,12 +4,13 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="default" sheetId="1" r:id="rId1"/>
+    <sheet name="relations" sheetId="2" r:id="rId1"/>
+    <sheet name="default" sheetId="1" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="162913" iterate="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -19,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="76">
   <si>
     <t>parameter</t>
   </si>
@@ -126,18 +127,6 @@
     <t>WASTE</t>
   </si>
   <si>
-    <t>FOOD TO CROP/BY- PRODUCTS</t>
-  </si>
-  <si>
-    <t>waste_household</t>
-  </si>
-  <si>
-    <t>waste_retail</t>
-  </si>
-  <si>
-    <t>waste_processing</t>
-  </si>
-  <si>
     <t>Wheat and products</t>
   </si>
   <si>
@@ -145,9 +134,6 @@
   </si>
   <si>
     <t>f_food</t>
-  </si>
-  <si>
-    <t>food_to_prod</t>
   </si>
   <si>
     <t>wheat</t>
@@ -224,11 +210,77 @@
   <si>
     <t>barley hulls</t>
   </si>
+  <si>
+    <t>food</t>
+  </si>
+  <si>
+    <t>food_group</t>
+  </si>
+  <si>
+    <t>f_waste_level</t>
+  </si>
+  <si>
+    <t>household</t>
+  </si>
+  <si>
+    <t>retail</t>
+  </si>
+  <si>
+    <t>processing</t>
+  </si>
+  <si>
+    <t>waste_share</t>
+  </si>
+  <si>
+    <t>Pig meat and products</t>
+  </si>
+  <si>
+    <t>meat</t>
+  </si>
+  <si>
+    <t>f_species</t>
+  </si>
+  <si>
+    <t>pigs</t>
+  </si>
+  <si>
+    <t>offals</t>
+  </si>
+  <si>
+    <t>fat</t>
+  </si>
+  <si>
+    <t>skins</t>
+  </si>
+  <si>
+    <t>butcher fat</t>
+  </si>
+  <si>
+    <r>
+      <t>CONVERSION FACTORS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (share of crop/animal product ending up as corresponding food or by-product)</t>
+    </r>
+  </si>
+  <si>
+    <t>conv_factor</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <numFmts count="1">
+    <numFmt numFmtId="171" formatCode="0.0"/>
+  </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -301,7 +353,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -311,6 +363,9 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="171" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -591,21 +646,75 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L51"/>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.28515625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>35</v>
+      </c>
+      <c r="B2" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>55</v>
+      </c>
+      <c r="B4" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>66</v>
+      </c>
+      <c r="B5" t="s">
+        <v>67</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:N60"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37.28515625" customWidth="1"/>
     <col min="2" max="2" width="19" customWidth="1"/>
-    <col min="3" max="4" width="15.42578125" customWidth="1"/>
-    <col min="5" max="7" width="14.28515625" customWidth="1"/>
-    <col min="8" max="8" width="21.42578125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="48.85546875" customWidth="1"/>
-    <col min="12" max="12" width="18.28515625" customWidth="1"/>
+    <col min="3" max="5" width="15.42578125" customWidth="1"/>
+    <col min="6" max="9" width="14.28515625" customWidth="1"/>
+    <col min="10" max="10" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="48.85546875" customWidth="1"/>
+    <col min="14" max="14" width="18.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>25</v>
@@ -614,34 +723,40 @@
         <v>27</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>40</v>
+        <v>68</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>56</v>
-      </c>
       <c r="G1" s="2" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="H1" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="J1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="I1" s="2" t="s">
+      <c r="K1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="2" t="s">
+      <c r="L1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="M1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="N1" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>17</v>
       </c>
@@ -651,31 +766,33 @@
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
-      <c r="H2" s="4"/>
-      <c r="I2" s="4"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
       <c r="J2" s="4"/>
       <c r="K2" s="4"/>
       <c r="L2" s="4"/>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="H3" t="s">
+      <c r="M2" s="4"/>
+      <c r="N2" s="4"/>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J3" t="s">
         <v>5</v>
       </c>
-      <c r="I3" s="1">
+      <c r="K3" s="1">
         <f>(5222847+5156448)/1000000</f>
         <v>10.379295000000001</v>
       </c>
-      <c r="J3" t="s">
+      <c r="L3" t="s">
         <v>6</v>
       </c>
-      <c r="K3" t="s">
+      <c r="M3" t="s">
         <v>8</v>
       </c>
-      <c r="L3" t="s">
+      <c r="N3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
         <v>9</v>
       </c>
@@ -685,13 +802,15 @@
       <c r="E5" s="3"/>
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
       <c r="J5" s="4"/>
       <c r="K5" s="4"/>
       <c r="L5" s="4"/>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M5" s="4"/>
+      <c r="N5" s="4"/>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>10</v>
       </c>
@@ -701,55 +820,57 @@
       <c r="E6" s="5"/>
       <c r="F6" s="5"/>
       <c r="G6" s="5"/>
-      <c r="H6" s="6"/>
-      <c r="I6" s="6"/>
+      <c r="H6" s="5"/>
+      <c r="I6" s="5"/>
       <c r="J6" s="6"/>
       <c r="K6" s="6"/>
       <c r="L6" s="6"/>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M6" s="6"/>
+      <c r="N6" s="6"/>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>39</v>
-      </c>
-      <c r="H7" t="s">
+        <v>35</v>
+      </c>
+      <c r="J7" t="s">
         <v>18</v>
       </c>
-      <c r="I7">
+      <c r="K7">
         <v>93.1</v>
       </c>
-      <c r="J7" t="s">
+      <c r="L7" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>51</v>
-      </c>
-      <c r="H8" t="s">
+        <v>46</v>
+      </c>
+      <c r="J8" t="s">
         <v>18</v>
       </c>
-      <c r="I8">
+      <c r="K8">
         <v>14.1</v>
       </c>
-      <c r="J8" t="s">
+      <c r="L8" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>60</v>
-      </c>
-      <c r="H9" t="s">
+        <v>55</v>
+      </c>
+      <c r="J9" t="s">
         <v>18</v>
       </c>
-      <c r="I9">
+      <c r="K9">
         <v>3.5</v>
       </c>
-      <c r="J9" t="s">
+      <c r="L9" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>11</v>
       </c>
@@ -759,13 +880,15 @@
       <c r="E10" s="5"/>
       <c r="F10" s="5"/>
       <c r="G10" s="5"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="5"/>
       <c r="J10" s="6"/>
       <c r="K10" s="6"/>
       <c r="L10" s="6"/>
-    </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M10" s="6"/>
+      <c r="N10" s="6"/>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>12</v>
       </c>
@@ -775,13 +898,15 @@
       <c r="E11" s="5"/>
       <c r="F11" s="5"/>
       <c r="G11" s="5"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="6"/>
+      <c r="H11" s="5"/>
+      <c r="I11" s="5"/>
       <c r="J11" s="6"/>
       <c r="K11" s="6"/>
       <c r="L11" s="6"/>
-    </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M11" s="6"/>
+      <c r="N11" s="6"/>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>13</v>
       </c>
@@ -791,13 +916,15 @@
       <c r="E12" s="5"/>
       <c r="F12" s="5"/>
       <c r="G12" s="5"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
+      <c r="H12" s="5"/>
+      <c r="I12" s="5"/>
       <c r="J12" s="6"/>
       <c r="K12" s="6"/>
       <c r="L12" s="6"/>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M12" s="6"/>
+      <c r="N12" s="6"/>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>14</v>
       </c>
@@ -807,13 +934,15 @@
       <c r="E13" s="5"/>
       <c r="F13" s="5"/>
       <c r="G13" s="5"/>
-      <c r="H13" s="6"/>
-      <c r="I13" s="6"/>
+      <c r="H13" s="5"/>
+      <c r="I13" s="5"/>
       <c r="J13" s="6"/>
       <c r="K13" s="6"/>
       <c r="L13" s="6"/>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M13" s="6"/>
+      <c r="N13" s="6"/>
+    </row>
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>23</v>
       </c>
@@ -823,31 +952,31 @@
       <c r="E14" s="5"/>
       <c r="F14" s="5"/>
       <c r="G14" s="5"/>
-      <c r="H14" s="6"/>
-      <c r="I14" s="6"/>
+      <c r="H14" s="5"/>
+      <c r="I14" s="5"/>
       <c r="J14" s="6"/>
       <c r="K14" s="6"/>
       <c r="L14" s="6"/>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A15" s="5" t="s">
+      <c r="M14" s="6"/>
+      <c r="N14" s="6"/>
+    </row>
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>66</v>
+      </c>
+      <c r="J15" t="s">
+        <v>18</v>
+      </c>
+      <c r="K15">
+        <v>60.6</v>
+      </c>
+      <c r="L15" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A16" s="5" t="s">
         <v>15</v>
-      </c>
-      <c r="B15" s="5"/>
-      <c r="C15" s="5"/>
-      <c r="D15" s="5"/>
-      <c r="E15" s="5"/>
-      <c r="F15" s="5"/>
-      <c r="G15" s="5"/>
-      <c r="H15" s="6"/>
-      <c r="I15" s="6"/>
-      <c r="J15" s="6"/>
-      <c r="K15" s="6"/>
-      <c r="L15" s="6"/>
-    </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A16" s="5" t="s">
-        <v>16</v>
       </c>
       <c r="B16" s="5"/>
       <c r="C16" s="5"/>
@@ -855,15 +984,17 @@
       <c r="E16" s="5"/>
       <c r="F16" s="5"/>
       <c r="G16" s="5"/>
-      <c r="H16" s="6"/>
-      <c r="I16" s="6"/>
+      <c r="H16" s="5"/>
+      <c r="I16" s="5"/>
       <c r="J16" s="6"/>
       <c r="K16" s="6"/>
       <c r="L16" s="6"/>
-    </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M16" s="6"/>
+      <c r="N16" s="6"/>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
@@ -871,15 +1002,17 @@
       <c r="E17" s="5"/>
       <c r="F17" s="5"/>
       <c r="G17" s="5"/>
-      <c r="H17" s="6"/>
-      <c r="I17" s="6"/>
+      <c r="H17" s="5"/>
+      <c r="I17" s="5"/>
       <c r="J17" s="6"/>
       <c r="K17" s="6"/>
       <c r="L17" s="6"/>
-    </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M17" s="6"/>
+      <c r="N17" s="6"/>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B18" s="5"/>
       <c r="C18" s="5"/>
@@ -887,15 +1020,17 @@
       <c r="E18" s="5"/>
       <c r="F18" s="5"/>
       <c r="G18" s="5"/>
-      <c r="H18" s="6"/>
-      <c r="I18" s="6"/>
+      <c r="H18" s="5"/>
+      <c r="I18" s="5"/>
       <c r="J18" s="6"/>
       <c r="K18" s="6"/>
       <c r="L18" s="6"/>
-    </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M18" s="6"/>
+      <c r="N18" s="6"/>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B19" s="5"/>
       <c r="C19" s="5"/>
@@ -903,15 +1038,17 @@
       <c r="E19" s="5"/>
       <c r="F19" s="5"/>
       <c r="G19" s="5"/>
-      <c r="H19" s="6"/>
-      <c r="I19" s="6"/>
+      <c r="H19" s="5"/>
+      <c r="I19" s="5"/>
       <c r="J19" s="6"/>
       <c r="K19" s="6"/>
       <c r="L19" s="6"/>
-    </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M19" s="6"/>
+      <c r="N19" s="6"/>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
@@ -919,15 +1056,17 @@
       <c r="E20" s="5"/>
       <c r="F20" s="5"/>
       <c r="G20" s="5"/>
-      <c r="H20" s="6"/>
-      <c r="I20" s="6"/>
+      <c r="H20" s="5"/>
+      <c r="I20" s="5"/>
       <c r="J20" s="6"/>
       <c r="K20" s="6"/>
       <c r="L20" s="6"/>
-    </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M20" s="6"/>
+      <c r="N20" s="6"/>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B21" s="5"/>
       <c r="C21" s="5"/>
@@ -935,15 +1074,17 @@
       <c r="E21" s="5"/>
       <c r="F21" s="5"/>
       <c r="G21" s="5"/>
-      <c r="H21" s="6"/>
-      <c r="I21" s="6"/>
+      <c r="H21" s="5"/>
+      <c r="I21" s="5"/>
       <c r="J21" s="6"/>
       <c r="K21" s="6"/>
       <c r="L21" s="6"/>
-    </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M21" s="6"/>
+      <c r="N21" s="6"/>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B22" s="5"/>
       <c r="C22" s="5"/>
@@ -951,15 +1092,17 @@
       <c r="E22" s="5"/>
       <c r="F22" s="5"/>
       <c r="G22" s="5"/>
-      <c r="H22" s="6"/>
-      <c r="I22" s="6"/>
+      <c r="H22" s="5"/>
+      <c r="I22" s="5"/>
       <c r="J22" s="6"/>
       <c r="K22" s="6"/>
       <c r="L22" s="6"/>
-    </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M22" s="6"/>
+      <c r="N22" s="6"/>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B23" s="5"/>
       <c r="C23" s="5"/>
@@ -967,15 +1110,17 @@
       <c r="E23" s="5"/>
       <c r="F23" s="5"/>
       <c r="G23" s="5"/>
-      <c r="H23" s="6"/>
-      <c r="I23" s="6"/>
+      <c r="H23" s="5"/>
+      <c r="I23" s="5"/>
       <c r="J23" s="6"/>
       <c r="K23" s="6"/>
       <c r="L23" s="6"/>
-    </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M23" s="6"/>
+      <c r="N23" s="6"/>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B24" s="5"/>
       <c r="C24" s="5"/>
@@ -983,15 +1128,17 @@
       <c r="E24" s="5"/>
       <c r="F24" s="5"/>
       <c r="G24" s="5"/>
-      <c r="H24" s="6"/>
-      <c r="I24" s="6"/>
+      <c r="H24" s="5"/>
+      <c r="I24" s="5"/>
       <c r="J24" s="6"/>
       <c r="K24" s="6"/>
       <c r="L24" s="6"/>
-    </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M24" s="6"/>
+      <c r="N24" s="6"/>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B25" s="5"/>
       <c r="C25" s="5"/>
@@ -999,363 +1146,640 @@
       <c r="E25" s="5"/>
       <c r="F25" s="5"/>
       <c r="G25" s="5"/>
-      <c r="H25" s="6"/>
-      <c r="I25" s="6"/>
+      <c r="H25" s="5"/>
+      <c r="I25" s="5"/>
       <c r="J25" s="6"/>
       <c r="K25" s="6"/>
       <c r="L25" s="6"/>
-    </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A27" s="3" t="s">
+      <c r="M25" s="6"/>
+      <c r="N25" s="6"/>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A26" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B26" s="5"/>
+      <c r="C26" s="5"/>
+      <c r="D26" s="5"/>
+      <c r="E26" s="5"/>
+      <c r="F26" s="5"/>
+      <c r="G26" s="5"/>
+      <c r="H26" s="5"/>
+      <c r="I26" s="5"/>
+      <c r="J26" s="6"/>
+      <c r="K26" s="6"/>
+      <c r="L26" s="6"/>
+      <c r="M26" s="6"/>
+      <c r="N26" s="6"/>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A28" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="B27" s="3"/>
-      <c r="C27" s="3"/>
-      <c r="D27" s="3"/>
-      <c r="E27" s="3"/>
-      <c r="F27" s="3"/>
-      <c r="G27" s="3"/>
-      <c r="H27" s="4"/>
-      <c r="I27" s="4"/>
-      <c r="J27" s="4"/>
-      <c r="K27" s="4"/>
-      <c r="L27" s="4"/>
-    </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A28" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B28" s="5"/>
-      <c r="C28" s="5"/>
-      <c r="D28" s="5"/>
-      <c r="E28" s="5"/>
-      <c r="F28" s="5"/>
-      <c r="G28" s="5"/>
-      <c r="H28" s="6"/>
-      <c r="I28" s="6"/>
-      <c r="J28" s="6"/>
-      <c r="K28" s="6"/>
-      <c r="L28" s="6"/>
-    </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="B28" s="3"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+      <c r="I28" s="3"/>
+      <c r="J28" s="4"/>
+      <c r="K28" s="4"/>
+      <c r="L28" s="4"/>
+      <c r="M28" s="4"/>
+      <c r="N28" s="4"/>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B29" t="s">
         <v>26</v>
       </c>
-      <c r="H29" t="s">
-        <v>36</v>
-      </c>
-      <c r="I29">
+      <c r="I29" t="s">
+        <v>62</v>
+      </c>
+      <c r="J29" t="s">
+        <v>65</v>
+      </c>
+      <c r="K29">
         <v>25</v>
       </c>
-      <c r="J29" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L29" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B30" t="s">
         <v>26</v>
       </c>
-      <c r="H30" t="s">
-        <v>37</v>
-      </c>
-      <c r="I30">
+      <c r="I30" t="s">
+        <v>63</v>
+      </c>
+      <c r="J30" t="s">
+        <v>65</v>
+      </c>
+      <c r="K30">
         <v>2</v>
       </c>
-      <c r="J30" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="L30" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B31" t="s">
         <v>26</v>
       </c>
-      <c r="H31" t="s">
+      <c r="I31" t="s">
+        <v>64</v>
+      </c>
+      <c r="J31" t="s">
+        <v>65</v>
+      </c>
+      <c r="K31" s="7">
+        <v>10.5</v>
+      </c>
+      <c r="L31" t="s">
+        <v>39</v>
+      </c>
+      <c r="M31" s="7" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B32" t="s">
+        <v>67</v>
+      </c>
+      <c r="I32" t="s">
+        <v>62</v>
+      </c>
+      <c r="J32" t="s">
+        <v>65</v>
+      </c>
+      <c r="K32">
+        <v>11</v>
+      </c>
+      <c r="L32" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B33" t="s">
+        <v>67</v>
+      </c>
+      <c r="I33" t="s">
+        <v>63</v>
+      </c>
+      <c r="J33" t="s">
+        <v>65</v>
+      </c>
+      <c r="K33">
+        <v>4</v>
+      </c>
+      <c r="L33" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="B34" t="s">
+        <v>67</v>
+      </c>
+      <c r="I34" t="s">
+        <v>64</v>
+      </c>
+      <c r="J34" t="s">
+        <v>65</v>
+      </c>
+      <c r="K34" s="7">
+        <v>5</v>
+      </c>
+      <c r="L34" t="s">
+        <v>39</v>
+      </c>
+      <c r="M34" s="7" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="36" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A36" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B36" s="3"/>
+      <c r="C36" s="3"/>
+      <c r="D36" s="3"/>
+      <c r="E36" s="3"/>
+      <c r="F36" s="3"/>
+      <c r="G36" s="3"/>
+      <c r="H36" s="3"/>
+      <c r="I36" s="3"/>
+      <c r="J36" s="4"/>
+      <c r="K36" s="4"/>
+      <c r="L36" s="4"/>
+      <c r="M36" s="4"/>
+      <c r="N36" s="4"/>
+    </row>
+    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>35</v>
+      </c>
+      <c r="C37" t="s">
         <v>38</v>
       </c>
-      <c r="I31">
-        <v>10.5</v>
-      </c>
-      <c r="J31" t="s">
+      <c r="J37" t="s">
+        <v>75</v>
+      </c>
+      <c r="K37">
+        <v>79</v>
+      </c>
+      <c r="L37" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="38" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>35</v>
+      </c>
+      <c r="F38" t="s">
         <v>44</v>
       </c>
-      <c r="K31" s="7" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A33" s="3" t="s">
+      <c r="J38" t="s">
+        <v>75</v>
+      </c>
+      <c r="K38">
+        <v>19</v>
+      </c>
+      <c r="L38" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="39" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
         <v>35</v>
       </c>
-      <c r="B33" s="3"/>
-      <c r="C33" s="3"/>
-      <c r="D33" s="3"/>
-      <c r="E33" s="3"/>
-      <c r="F33" s="3"/>
-      <c r="G33" s="3"/>
-      <c r="H33" s="4"/>
-      <c r="I33" s="4"/>
-      <c r="J33" s="4"/>
-      <c r="K33" s="4"/>
-      <c r="L33" s="4"/>
-    </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>39</v>
-      </c>
-      <c r="C34" t="s">
-        <v>43</v>
-      </c>
-      <c r="H34" t="s">
+      <c r="F39" t="s">
+        <v>45</v>
+      </c>
+      <c r="J39" t="s">
+        <v>75</v>
+      </c>
+      <c r="K39">
+        <v>2</v>
+      </c>
+      <c r="L39" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="40" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A40" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B40" s="9"/>
+      <c r="C40" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="D40" s="9"/>
+      <c r="E40" s="9"/>
+      <c r="F40" s="9"/>
+      <c r="G40" s="9"/>
+      <c r="H40" s="9"/>
+      <c r="I40" s="9"/>
+      <c r="J40" t="s">
+        <v>75</v>
+      </c>
+      <c r="K40" s="9">
+        <v>91</v>
+      </c>
+      <c r="L40" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="M40" s="9"/>
+      <c r="N40" s="9"/>
+    </row>
+    <row r="41" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A41" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B41" s="9"/>
+      <c r="C41" s="9"/>
+      <c r="D41" s="9"/>
+      <c r="E41" s="9"/>
+      <c r="F41" s="9" t="s">
+        <v>57</v>
+      </c>
+      <c r="G41" s="9"/>
+      <c r="H41" s="9"/>
+      <c r="I41" s="9"/>
+      <c r="J41" t="s">
+        <v>75</v>
+      </c>
+      <c r="K41" s="9">
+        <v>0</v>
+      </c>
+      <c r="L41" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="M41" s="9"/>
+      <c r="N41" s="9"/>
+    </row>
+    <row r="42" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A42" s="9" t="s">
+        <v>55</v>
+      </c>
+      <c r="B42" s="9"/>
+      <c r="C42" s="9"/>
+      <c r="D42" s="9"/>
+      <c r="E42" s="9"/>
+      <c r="F42" s="9" t="s">
+        <v>58</v>
+      </c>
+      <c r="G42" s="9"/>
+      <c r="H42" s="9"/>
+      <c r="I42" s="9"/>
+      <c r="J42" t="s">
+        <v>75</v>
+      </c>
+      <c r="K42" s="9">
+        <v>9</v>
+      </c>
+      <c r="L42" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="M42" s="9"/>
+      <c r="N42" s="9"/>
+    </row>
+    <row r="43" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A43" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="B43" s="9"/>
+      <c r="C43" s="9"/>
+      <c r="D43" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="E43" s="9" t="s">
+        <v>67</v>
+      </c>
+      <c r="F43" s="9"/>
+      <c r="G43" s="9"/>
+      <c r="H43" s="9"/>
+      <c r="I43" s="9"/>
+      <c r="J43" t="s">
+        <v>75</v>
+      </c>
+      <c r="K43" s="10">
+        <v>73</v>
+      </c>
+      <c r="L43" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="M43" s="9"/>
+      <c r="N43" s="9"/>
+    </row>
+    <row r="44" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A44" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="B44" s="9"/>
+      <c r="C44" s="9"/>
+      <c r="D44" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="E44" s="9"/>
+      <c r="F44" s="9" t="s">
+        <v>70</v>
+      </c>
+      <c r="G44" s="9"/>
+      <c r="H44" s="9"/>
+      <c r="I44" s="9"/>
+      <c r="J44" t="s">
+        <v>75</v>
+      </c>
+      <c r="K44" s="11">
+        <f>(1/0.76)*4</f>
+        <v>5.2631578947368425</v>
+      </c>
+      <c r="L44" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="M44" s="9"/>
+      <c r="N44" s="9"/>
+    </row>
+    <row r="45" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A45" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="B45" s="9"/>
+      <c r="C45" s="9"/>
+      <c r="D45" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="E45" s="9"/>
+      <c r="F45" s="9" t="s">
+        <v>71</v>
+      </c>
+      <c r="G45" s="9"/>
+      <c r="H45" s="9"/>
+      <c r="I45" s="9"/>
+      <c r="J45" t="s">
+        <v>75</v>
+      </c>
+      <c r="K45" s="11">
+        <f>(1/0.76)*6</f>
+        <v>7.8947368421052637</v>
+      </c>
+      <c r="L45" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="M45" s="9"/>
+      <c r="N45" s="9"/>
+    </row>
+    <row r="46" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A46" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="B46" s="9"/>
+      <c r="C46" s="9"/>
+      <c r="D46" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="E46" s="9"/>
+      <c r="F46" s="9" t="s">
+        <v>72</v>
+      </c>
+      <c r="G46" s="9"/>
+      <c r="H46" s="9"/>
+      <c r="I46" s="9"/>
+      <c r="J46" t="s">
+        <v>75</v>
+      </c>
+      <c r="K46" s="11">
+        <f>(1/0.76)*5</f>
+        <v>6.5789473684210531</v>
+      </c>
+      <c r="L46" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="M46" s="9"/>
+      <c r="N46" s="9"/>
+    </row>
+    <row r="47" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A47" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="B47" s="9"/>
+      <c r="C47" s="9"/>
+      <c r="D47" s="9" t="s">
+        <v>69</v>
+      </c>
+      <c r="E47" s="9"/>
+      <c r="F47" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="G47" s="9"/>
+      <c r="H47" s="9"/>
+      <c r="I47" s="9"/>
+      <c r="J47" t="s">
+        <v>75</v>
+      </c>
+      <c r="K47" s="10">
+        <v>18</v>
+      </c>
+      <c r="L47" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="M47" s="9"/>
+      <c r="N47" s="9"/>
+    </row>
+    <row r="48" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A48" s="9"/>
+      <c r="B48" s="9"/>
+      <c r="C48" s="9"/>
+      <c r="D48" s="9"/>
+      <c r="E48" s="9"/>
+      <c r="F48" s="9"/>
+      <c r="G48" s="9"/>
+      <c r="H48" s="9"/>
+      <c r="I48" s="9"/>
+      <c r="J48" s="9"/>
+      <c r="K48" s="9"/>
+      <c r="L48" s="9"/>
+      <c r="M48" s="9"/>
+      <c r="N48" s="9"/>
+    </row>
+    <row r="49" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A49" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B49" s="3"/>
+      <c r="C49" s="3"/>
+      <c r="D49" s="3"/>
+      <c r="E49" s="3"/>
+      <c r="F49" s="3"/>
+      <c r="G49" s="3"/>
+      <c r="H49" s="3"/>
+      <c r="I49" s="3"/>
+      <c r="J49" s="4"/>
+      <c r="K49" s="4"/>
+      <c r="L49" s="4"/>
+      <c r="M49" s="4"/>
+      <c r="N49" s="4"/>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J50" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="K50" s="8">
+        <v>100</v>
+      </c>
+      <c r="L50" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="M50" s="8" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>35</v>
+      </c>
+      <c r="J51" t="s">
+        <v>41</v>
+      </c>
+      <c r="K51">
+        <v>22</v>
+      </c>
+      <c r="L51" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>46</v>
+      </c>
+      <c r="J52" t="s">
+        <v>41</v>
+      </c>
+      <c r="K52">
+        <v>100</v>
+      </c>
+      <c r="L52" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>55</v>
+      </c>
+      <c r="J53" t="s">
+        <v>41</v>
+      </c>
+      <c r="K53">
+        <v>4</v>
+      </c>
+      <c r="L53" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>66</v>
+      </c>
+      <c r="J54" t="s">
+        <v>41</v>
+      </c>
+      <c r="K54">
+        <v>36</v>
+      </c>
+      <c r="L54" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A56" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="B56" s="3"/>
+      <c r="C56" s="3"/>
+      <c r="D56" s="3"/>
+      <c r="E56" s="3"/>
+      <c r="F56" s="3"/>
+      <c r="G56" s="3"/>
+      <c r="H56" s="3"/>
+      <c r="I56" s="3"/>
+      <c r="J56" s="4"/>
+      <c r="K56" s="4"/>
+      <c r="L56" s="4"/>
+      <c r="M56" s="4"/>
+      <c r="N56" s="4"/>
+    </row>
+    <row r="57" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="G57" s="8"/>
+      <c r="H57" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="I57" s="8"/>
+      <c r="J57" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="I34">
-        <v>79</v>
-      </c>
-      <c r="J34" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>39</v>
-      </c>
-      <c r="E35" t="s">
-        <v>49</v>
-      </c>
-      <c r="H35" t="s">
+      <c r="K57" s="8">
+        <v>-100</v>
+      </c>
+      <c r="L57" s="8" t="s">
+        <v>50</v>
+      </c>
+      <c r="M57" s="8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="58" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="G58" s="8"/>
+      <c r="H58" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="I58" s="8"/>
+      <c r="J58" s="8" t="s">
         <v>42</v>
       </c>
-      <c r="I35">
-        <v>19</v>
-      </c>
-      <c r="J35" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>39</v>
-      </c>
-      <c r="E36" t="s">
-        <v>50</v>
-      </c>
-      <c r="H36" t="s">
+      <c r="K58" s="8">
+        <v>0</v>
+      </c>
+      <c r="L58" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="M58" s="8" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="59" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>35</v>
+      </c>
+      <c r="H59" t="s">
+        <v>47</v>
+      </c>
+      <c r="J59" t="s">
         <v>42</v>
       </c>
-      <c r="I36">
-        <v>2</v>
-      </c>
-      <c r="J36" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>60</v>
-      </c>
-      <c r="C37" t="s">
-        <v>61</v>
-      </c>
-      <c r="H37" t="s">
+      <c r="K59" s="7">
+        <v>5</v>
+      </c>
+      <c r="L59" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="60" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>55</v>
+      </c>
+      <c r="H60" t="s">
+        <v>47</v>
+      </c>
+      <c r="J60" t="s">
         <v>42</v>
       </c>
-      <c r="I37">
-        <v>91</v>
-      </c>
-      <c r="J37" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>60</v>
-      </c>
-      <c r="E38" t="s">
-        <v>62</v>
-      </c>
-      <c r="H38" t="s">
-        <v>42</v>
-      </c>
-      <c r="I38">
-        <v>0</v>
-      </c>
-      <c r="J38" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>60</v>
-      </c>
-      <c r="E39" t="s">
-        <v>63</v>
-      </c>
-      <c r="H39" t="s">
-        <v>42</v>
-      </c>
-      <c r="I39">
-        <v>9</v>
-      </c>
-      <c r="J39" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A41" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="B41" s="3"/>
-      <c r="C41" s="3"/>
-      <c r="D41" s="3"/>
-      <c r="E41" s="3"/>
-      <c r="F41" s="3"/>
-      <c r="G41" s="3"/>
-      <c r="H41" s="4"/>
-      <c r="I41" s="4"/>
-      <c r="J41" s="4"/>
-      <c r="K41" s="4"/>
-      <c r="L41" s="4"/>
-    </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="H42" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="I42" s="8">
-        <v>100</v>
-      </c>
-      <c r="J42" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="K42" s="8" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>39</v>
-      </c>
-      <c r="H43" t="s">
-        <v>46</v>
-      </c>
-      <c r="I43">
-        <v>22</v>
-      </c>
-      <c r="J43" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>51</v>
-      </c>
-      <c r="H44" t="s">
-        <v>46</v>
-      </c>
-      <c r="I44">
-        <v>100</v>
-      </c>
-      <c r="J44" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>60</v>
-      </c>
-      <c r="H45" t="s">
-        <v>46</v>
-      </c>
-      <c r="I45">
-        <v>4</v>
-      </c>
-      <c r="J45" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A47" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="B47" s="3"/>
-      <c r="C47" s="3"/>
-      <c r="D47" s="3"/>
-      <c r="E47" s="3"/>
-      <c r="F47" s="3"/>
-      <c r="G47" s="3"/>
-      <c r="H47" s="4"/>
-      <c r="I47" s="4"/>
-      <c r="J47" s="4"/>
-      <c r="K47" s="4"/>
-      <c r="L47" s="4"/>
-    </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="F48" s="8"/>
-      <c r="G48" s="8" t="s">
-        <v>54</v>
-      </c>
-      <c r="H48" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="I48" s="8">
-        <v>-100</v>
-      </c>
-      <c r="J48" s="8" t="s">
-        <v>55</v>
-      </c>
-      <c r="K48" s="8" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="F49" s="8"/>
-      <c r="G49" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="H49" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="I49" s="8">
-        <v>0</v>
-      </c>
-      <c r="J49" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="K49" s="8" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>39</v>
-      </c>
-      <c r="G50" t="s">
-        <v>52</v>
-      </c>
-      <c r="H50" t="s">
-        <v>47</v>
-      </c>
-      <c r="I50" s="7">
-        <v>5</v>
-      </c>
-      <c r="J50" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>60</v>
-      </c>
-      <c r="G51" t="s">
-        <v>52</v>
-      </c>
-      <c r="H51" t="s">
-        <v>47</v>
-      </c>
-      <c r="I51" s="7">
+      <c r="K60" s="7">
         <v>10</v>
       </c>
-      <c r="J51" t="s">
-        <v>44</v>
+      <c r="L60" t="s">
+        <v>39</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implemented method for handling demand for seeds
</commit_message>
<xml_diff>
--- a/data/prod_parameters/Diet.xlsx
+++ b/data/prod_parameters/Diet.xlsx
@@ -8,6 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="default" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913" iterate="1"/>
   <extLst>
@@ -19,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="842" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="892" uniqueCount="196">
   <si>
     <t>parameter</t>
   </si>
@@ -303,9 +304,6 @@
     <t>conv_factor_by</t>
   </si>
   <si>
-    <t>Share conventional is calculated as what remains (value should be -100)</t>
-  </si>
-  <si>
     <t>domestic</t>
   </si>
   <si>
@@ -342,9 +340,6 @@
     <t>SJV stat</t>
   </si>
   <si>
-    <t>Share organic raw milk to dairies. Using product level shares difficult</t>
-  </si>
-  <si>
     <t>Bovine meat and products</t>
   </si>
   <si>
@@ -381,12 +376,6 @@
     <t>where do we handle discarded potatoes?</t>
   </si>
   <si>
-    <t>what is the remaining 81% ?</t>
-  </si>
-  <si>
-    <t>Is this from starch potatoes what is the remaining 80% ?</t>
-  </si>
-  <si>
     <t>potatoes table</t>
   </si>
   <si>
@@ -489,7 +478,61 @@
     <t>calc. based on 45.5% fat in seed and 20% fat in cold pressed cake</t>
   </si>
   <si>
-    <t>38% in Hannas sheet. what is remaining 2% ???</t>
+    <t>1/3 of oil other added here</t>
+  </si>
+  <si>
+    <t>Sunflowerseed oil and products</t>
+  </si>
+  <si>
+    <t>Olive oil and products</t>
+  </si>
+  <si>
+    <t>Carrots and turnips</t>
+  </si>
+  <si>
+    <t>carrots</t>
+  </si>
+  <si>
+    <t>Cabbages (and cauliflower &amp; broccoli)</t>
+  </si>
+  <si>
+    <t>Lettuce and spinach</t>
+  </si>
+  <si>
+    <t>Pumpkins, squash and gourds</t>
+  </si>
+  <si>
+    <t>Peas, green</t>
+  </si>
+  <si>
+    <t>Onions, dry</t>
+  </si>
+  <si>
+    <t>peas green</t>
+  </si>
+  <si>
+    <t>cabbages etc</t>
+  </si>
+  <si>
+    <t>lettuce and spinach</t>
+  </si>
+  <si>
+    <t>pumpkins and squash</t>
+  </si>
+  <si>
+    <t>other vegetables</t>
+  </si>
+  <si>
+    <t>onions</t>
+  </si>
+  <si>
+    <t>Other vegetables</t>
+  </si>
+  <si>
+    <t>assumed same as wheat</t>
+  </si>
+  <si>
+    <t>100% in Hanna's sheet</t>
   </si>
   <si>
     <r>
@@ -503,78 +546,92 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> (shares can be different for 'domestic' and 'imported' by specifying 'f_origin') </t>
+      <t xml:space="preserve"> (shares can be different for 'domestic' and 'imported' by specifying 'f_origin')</t>
     </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>0% organic fails FIX!!!!</t>
-    </r>
-  </si>
-  <si>
-    <t>1/3 of oil other added here</t>
-  </si>
-  <si>
-    <t>Sunflowerseed oil and products</t>
-  </si>
-  <si>
-    <t>Olive oil and products</t>
-  </si>
-  <si>
-    <t>Carrots and turnips</t>
-  </si>
-  <si>
-    <t>carrots</t>
-  </si>
-  <si>
-    <t>Cabbages (and cauliflower &amp; broccoli)</t>
-  </si>
-  <si>
-    <t>Lettuce and spinach</t>
-  </si>
-  <si>
-    <t>Pumpkins, squash and gourds</t>
-  </si>
-  <si>
-    <t>Peas, green</t>
-  </si>
-  <si>
-    <t>Onions, dry</t>
-  </si>
-  <si>
-    <t>peas green</t>
-  </si>
-  <si>
-    <t>cabbages etc</t>
-  </si>
-  <si>
-    <t>lettuce and spinach</t>
-  </si>
-  <si>
-    <t>pumpkins and squash</t>
-  </si>
-  <si>
-    <t>other vegetables</t>
-  </si>
-  <si>
-    <t>onions</t>
-  </si>
-  <si>
-    <t>Other vegetables</t>
-  </si>
-  <si>
-    <t>assumed same as wheat</t>
-  </si>
-  <si>
-    <t>54% in Hanna's sheet</t>
-  </si>
-  <si>
-    <t>100% in Hanna's sheet</t>
+  </si>
+  <si>
+    <t>Raps</t>
+  </si>
+  <si>
+    <t>Kanske används lite I FAME. Troligen ej I HVO</t>
+  </si>
+  <si>
+    <t>Kan vara annat, såpa</t>
+  </si>
+  <si>
+    <t>Margarin, Hanna kollar</t>
+  </si>
+  <si>
+    <t>Hönsen?</t>
+  </si>
+  <si>
+    <t>Fiskfoder? Export till Norge?</t>
+  </si>
+  <si>
+    <t>Potatis stärkelse</t>
+  </si>
+  <si>
+    <t>Konsumption kan vara underskattad</t>
+  </si>
+  <si>
+    <t>Finns det export</t>
+  </si>
+  <si>
+    <t>Vete</t>
+  </si>
+  <si>
+    <t>200 000 ton foder</t>
+  </si>
+  <si>
+    <t>600 000 ton spannmål (absolut majoritet vete) per år till Agroetanol. Även lite rågvete</t>
+  </si>
+  <si>
+    <t>Morötter</t>
+  </si>
+  <si>
+    <t>Morötter till foder</t>
+  </si>
+  <si>
+    <t>Avg. of "Klass 1&amp;2" and "Klass 3"</t>
+  </si>
+  <si>
+    <t>Ekologiska årsrapporten 2021</t>
+  </si>
+  <si>
+    <t>From share organic raw milk to dairies. Using product level shares difficult</t>
+  </si>
+  <si>
+    <t>From prod. stat</t>
+  </si>
+  <si>
+    <t>"Havregryn"</t>
+  </si>
+  <si>
+    <t>"Sallat"</t>
+  </si>
+  <si>
+    <t>"Morötter"</t>
+  </si>
+  <si>
+    <t>"Lök"</t>
+  </si>
+  <si>
+    <t>"Gurka"</t>
+  </si>
+  <si>
+    <t>"Tomater"</t>
+  </si>
+  <si>
+    <t>add protein by-prod</t>
+  </si>
+  <si>
+    <t>barley malt culms</t>
+  </si>
+  <si>
+    <t>maltgroddar</t>
+  </si>
+  <si>
+    <t>Share conventional is calculated as what remains (value should be -100). Do not specify per food</t>
   </si>
 </sst>
 </file>
@@ -584,7 +641,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -629,6 +686,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -662,7 +726,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -689,6 +753,8 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -969,7 +1035,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N216"/>
+  <dimension ref="A1:N221"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="37.28515625" customWidth="1"/>
@@ -1115,7 +1181,7 @@
         <v>19</v>
       </c>
       <c r="M7" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
@@ -1153,12 +1219,12 @@
         <v>19</v>
       </c>
       <c r="M9" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B10" t="s">
         <v>26</v>
@@ -1175,7 +1241,7 @@
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B11" t="s">
         <v>26</v>
@@ -1190,12 +1256,12 @@
         <v>19</v>
       </c>
       <c r="M11" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B12" t="s">
         <v>26</v>
@@ -1210,12 +1276,12 @@
         <v>19</v>
       </c>
       <c r="M12" s="7" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B13" t="s">
         <v>26</v>
@@ -1230,7 +1296,7 @@
         <v>19</v>
       </c>
       <c r="M13" s="7" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="14" spans="1:14" x14ac:dyDescent="0.25">
@@ -1253,10 +1319,10 @@
     </row>
     <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B15" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="J15" t="s">
         <v>18</v>
@@ -1270,10 +1336,10 @@
     </row>
     <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B16" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="J16" t="s">
         <v>18</v>
@@ -1287,10 +1353,10 @@
     </row>
     <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
+        <v>110</v>
+      </c>
+      <c r="B17" t="s">
         <v>112</v>
-      </c>
-      <c r="B17" t="s">
-        <v>114</v>
       </c>
       <c r="J17" t="s">
         <v>18</v>
@@ -1302,15 +1368,15 @@
         <v>19</v>
       </c>
       <c r="M17" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B18" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="J18" t="s">
         <v>18</v>
@@ -1342,10 +1408,10 @@
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" s="18" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="B20" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="J20" t="s">
         <v>18</v>
@@ -1359,10 +1425,10 @@
     </row>
     <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" s="18" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="B21" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="J21" t="s">
         <v>18</v>
@@ -1376,10 +1442,10 @@
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" s="18" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="B22" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="J22" t="s">
         <v>18</v>
@@ -1393,10 +1459,10 @@
     </row>
     <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" s="18" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="B23" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="J23" t="s">
         <v>18</v>
@@ -1410,10 +1476,10 @@
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" s="18" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="B24" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="J24" t="s">
         <v>18</v>
@@ -1427,10 +1493,10 @@
     </row>
     <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="18" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="B25" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="J25" t="s">
         <v>18</v>
@@ -1444,10 +1510,10 @@
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="18" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="B26" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="J26" t="s">
         <v>18</v>
@@ -1460,11 +1526,11 @@
       </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A27" s="7" t="s">
-        <v>123</v>
+      <c r="A27" s="18" t="s">
+        <v>119</v>
       </c>
       <c r="B27" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="J27" t="s">
         <v>18</v>
@@ -1478,10 +1544,10 @@
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="18" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="B28" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="J28" t="s">
         <v>18</v>
@@ -1731,7 +1797,7 @@
     </row>
     <row r="42" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B42" t="s">
         <v>58</v>
@@ -1838,31 +1904,31 @@
     </row>
     <row r="48" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="B48" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="J48" t="s">
         <v>18</v>
       </c>
       <c r="K48" s="23">
-        <f>6+4.4/3</f>
-        <v>7.4666666666666668</v>
+        <f>6+4.4/3+13</f>
+        <v>20.466666666666669</v>
       </c>
       <c r="L48" t="s">
         <v>19</v>
       </c>
       <c r="M48" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
     </row>
     <row r="49" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="B49" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="J49" t="s">
         <v>18</v>
@@ -1875,15 +1941,15 @@
         <v>19</v>
       </c>
       <c r="M49" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
     </row>
     <row r="50" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="B50" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="J50" t="s">
         <v>18</v>
@@ -1896,7 +1962,7 @@
         <v>19</v>
       </c>
       <c r="M50" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.25">
@@ -1937,10 +2003,10 @@
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B53" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="J53" t="s">
         <v>18</v>
@@ -2093,12 +2159,12 @@
         <v>39</v>
       </c>
       <c r="M62" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="63" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B63" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I63" t="s">
         <v>53</v>
@@ -2115,7 +2181,7 @@
     </row>
     <row r="64" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B64" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I64" t="s">
         <v>54</v>
@@ -2132,7 +2198,7 @@
     </row>
     <row r="65" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B65" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="I65" t="s">
         <v>55</v>
@@ -2147,12 +2213,12 @@
         <v>39</v>
       </c>
       <c r="M65" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="66" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B66" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="I66" t="s">
         <v>53</v>
@@ -2169,7 +2235,7 @@
     </row>
     <row r="67" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B67" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="I67" t="s">
         <v>54</v>
@@ -2186,7 +2252,7 @@
     </row>
     <row r="68" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B68" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="I68" t="s">
         <v>55</v>
@@ -2201,7 +2267,7 @@
         <v>39</v>
       </c>
       <c r="M68" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="69" spans="2:13" x14ac:dyDescent="0.25">
@@ -2256,7 +2322,7 @@
         <v>39</v>
       </c>
       <c r="M71" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="72" spans="2:13" x14ac:dyDescent="0.25">
@@ -2310,12 +2376,12 @@
         <v>39</v>
       </c>
       <c r="M74" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="75" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B75" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="I75" t="s">
         <v>53</v>
@@ -2332,7 +2398,7 @@
     </row>
     <row r="76" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B76" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="I76" t="s">
         <v>54</v>
@@ -2349,7 +2415,7 @@
     </row>
     <row r="77" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B77" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="I77" t="s">
         <v>55</v>
@@ -2364,12 +2430,12 @@
         <v>39</v>
       </c>
       <c r="M77" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="78" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B78" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="I78" t="s">
         <v>53</v>
@@ -2386,7 +2452,7 @@
     </row>
     <row r="79" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B79" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="I79" t="s">
         <v>54</v>
@@ -2403,7 +2469,7 @@
     </row>
     <row r="80" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B80" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="I80" t="s">
         <v>55</v>
@@ -2418,7 +2484,7 @@
         <v>39</v>
       </c>
       <c r="M80" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="82" spans="1:14" x14ac:dyDescent="0.25">
@@ -2502,7 +2568,7 @@
         <v>39</v>
       </c>
       <c r="N86" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="87" spans="1:14" x14ac:dyDescent="0.25">
@@ -2513,7 +2579,7 @@
         <v>38</v>
       </c>
       <c r="F87" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="J87" t="s">
         <v>89</v>
@@ -2525,7 +2591,7 @@
         <v>39</v>
       </c>
       <c r="N87" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="88" spans="1:14" x14ac:dyDescent="0.25">
@@ -2536,7 +2602,7 @@
         <v>38</v>
       </c>
       <c r="F88" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="J88" t="s">
         <v>89</v>
@@ -2548,7 +2614,7 @@
         <v>39</v>
       </c>
       <c r="N88" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="89" spans="1:14" x14ac:dyDescent="0.25">
@@ -2576,7 +2642,7 @@
       </c>
       <c r="M89" s="9"/>
       <c r="N89" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="90" spans="1:14" x14ac:dyDescent="0.25">
@@ -2590,7 +2656,7 @@
       <c r="D90" s="9"/>
       <c r="E90" s="9"/>
       <c r="F90" s="9" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="G90" s="9"/>
       <c r="H90" s="9"/>
@@ -2606,7 +2672,7 @@
       </c>
       <c r="M90" s="9"/>
       <c r="N90" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="91" spans="1:14" x14ac:dyDescent="0.25">
@@ -2620,7 +2686,7 @@
       <c r="D91" s="9"/>
       <c r="E91" s="9"/>
       <c r="F91" s="9" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
       <c r="G91" s="9"/>
       <c r="H91" s="9"/>
@@ -2636,16 +2702,16 @@
       </c>
       <c r="M91" s="9"/>
       <c r="N91" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="92" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B92" s="9"/>
       <c r="C92" s="10" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D92" s="9"/>
       <c r="E92" s="9"/>
@@ -2664,21 +2730,21 @@
       </c>
       <c r="M92" s="9"/>
       <c r="N92" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="93" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B93" s="9"/>
       <c r="C93" s="10" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D93" s="9"/>
       <c r="E93" s="9"/>
       <c r="F93" s="10" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="G93" s="9"/>
       <c r="H93" s="9"/>
@@ -2694,16 +2760,16 @@
       </c>
       <c r="M93" s="9"/>
       <c r="N93" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="94" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B94" s="9"/>
       <c r="C94" s="10" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D94" s="9"/>
       <c r="E94" s="9"/>
@@ -2722,21 +2788,21 @@
       </c>
       <c r="M94" s="9"/>
       <c r="N94" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="95" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B95" s="9"/>
       <c r="C95" s="10" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D95" s="9"/>
       <c r="E95" s="9"/>
       <c r="F95" s="10" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
       <c r="G95" s="9"/>
       <c r="H95" s="9"/>
@@ -2752,7 +2818,7 @@
       </c>
       <c r="M95" s="9"/>
       <c r="N95" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="96" spans="1:14" x14ac:dyDescent="0.25">
@@ -2775,11 +2841,11 @@
     </row>
     <row r="97" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A97" s="7" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B97" s="9"/>
       <c r="C97" s="10" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="D97" s="9"/>
       <c r="E97" s="9"/>
@@ -2797,16 +2863,16 @@
         <v>39</v>
       </c>
       <c r="M97" s="11" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="98" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A98" s="7" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B98" s="9"/>
       <c r="C98" s="10" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="D98" s="9"/>
       <c r="E98" s="9"/>
@@ -2827,16 +2893,16 @@
     </row>
     <row r="99" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A99" s="7" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B99" s="9"/>
       <c r="C99" s="10" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="D99" s="9"/>
       <c r="E99" s="9"/>
       <c r="F99" s="10" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="G99" s="9"/>
       <c r="H99" s="9"/>
@@ -2854,11 +2920,11 @@
     </row>
     <row r="100" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A100" s="7" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B100" s="9"/>
       <c r="C100" s="12" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="D100" s="9"/>
       <c r="E100" s="9"/>
@@ -2876,16 +2942,16 @@
         <v>39</v>
       </c>
       <c r="M100" s="11" t="s">
-        <v>117</v>
+        <v>192</v>
       </c>
     </row>
     <row r="101" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A101" s="7" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B101" s="9"/>
       <c r="C101" s="10" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="D101" s="9"/>
       <c r="E101" s="9"/>
@@ -2903,7 +2969,7 @@
         <v>39</v>
       </c>
       <c r="M101" s="11" t="s">
-        <v>116</v>
+        <v>192</v>
       </c>
     </row>
     <row r="102" spans="1:14" x14ac:dyDescent="0.25">
@@ -2926,10 +2992,10 @@
     </row>
     <row r="103" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A103" s="18" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="C103" s="10" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="J103" t="s">
         <v>88</v>
@@ -2943,10 +3009,10 @@
     </row>
     <row r="104" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A104" s="18" t="s">
+        <v>157</v>
+      </c>
+      <c r="C104" s="10" t="s">
         <v>163</v>
-      </c>
-      <c r="C104" s="10" t="s">
-        <v>169</v>
       </c>
       <c r="J104" t="s">
         <v>88</v>
@@ -2960,10 +3026,10 @@
     </row>
     <row r="105" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A105" s="18" t="s">
+        <v>153</v>
+      </c>
+      <c r="C105" s="10" t="s">
         <v>159</v>
-      </c>
-      <c r="C105" s="10" t="s">
-        <v>165</v>
       </c>
       <c r="J105" t="s">
         <v>88</v>
@@ -2977,10 +3043,10 @@
     </row>
     <row r="106" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A106" s="18" t="s">
+        <v>154</v>
+      </c>
+      <c r="C106" s="10" t="s">
         <v>160</v>
-      </c>
-      <c r="C106" s="10" t="s">
-        <v>166</v>
       </c>
       <c r="J106" t="s">
         <v>88</v>
@@ -2994,10 +3060,10 @@
     </row>
     <row r="107" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A107" s="18" t="s">
+        <v>155</v>
+      </c>
+      <c r="C107" s="10" t="s">
         <v>161</v>
-      </c>
-      <c r="C107" s="10" t="s">
-        <v>167</v>
       </c>
       <c r="J107" t="s">
         <v>88</v>
@@ -3011,10 +3077,10 @@
     </row>
     <row r="108" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A108" s="18" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="C108" s="10" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="J108" t="s">
         <v>88</v>
@@ -3028,11 +3094,11 @@
     </row>
     <row r="109" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A109" s="18" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="B109" s="9"/>
       <c r="C109" s="10" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="D109" s="9"/>
       <c r="E109" s="9"/>
@@ -3052,12 +3118,12 @@
       <c r="M109" s="11"/>
     </row>
     <row r="110" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A110" s="7" t="s">
-        <v>123</v>
+      <c r="A110" s="18" t="s">
+        <v>119</v>
       </c>
       <c r="B110" s="9"/>
       <c r="C110" s="10" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="D110" s="9"/>
       <c r="E110" s="9"/>
@@ -3078,11 +3144,11 @@
     </row>
     <row r="111" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A111" s="18" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="B111" s="9"/>
       <c r="C111" s="10" t="s">
-        <v>168</v>
+        <v>162</v>
       </c>
       <c r="D111" s="9"/>
       <c r="E111" s="9"/>
@@ -3149,7 +3215,7 @@
         <v>74</v>
       </c>
       <c r="N113" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="114" spans="1:14" x14ac:dyDescent="0.25">
@@ -3181,7 +3247,7 @@
         <v>39</v>
       </c>
       <c r="N114" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="115" spans="1:14" x14ac:dyDescent="0.25">
@@ -3214,7 +3280,7 @@
         <v>75</v>
       </c>
       <c r="N115" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="116" spans="1:14" x14ac:dyDescent="0.25">
@@ -3246,7 +3312,7 @@
         <v>39</v>
       </c>
       <c r="N116" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="117" spans="1:14" x14ac:dyDescent="0.25">
@@ -3279,7 +3345,7 @@
         <v>76</v>
       </c>
       <c r="N117" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="118" spans="1:14" x14ac:dyDescent="0.25">
@@ -3311,7 +3377,7 @@
         <v>39</v>
       </c>
       <c r="N118" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="119" spans="1:14" x14ac:dyDescent="0.25">
@@ -3344,7 +3410,7 @@
         <v>83</v>
       </c>
       <c r="N119" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="120" spans="1:14" x14ac:dyDescent="0.25">
@@ -3376,7 +3442,7 @@
         <v>39</v>
       </c>
       <c r="N120" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="121" spans="1:14" x14ac:dyDescent="0.25">
@@ -3408,7 +3474,7 @@
         <v>39</v>
       </c>
       <c r="N121" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="122" spans="1:14" x14ac:dyDescent="0.25">
@@ -3441,7 +3507,7 @@
         <v>81</v>
       </c>
       <c r="N122" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="123" spans="1:14" x14ac:dyDescent="0.25">
@@ -3474,7 +3540,7 @@
         <v>77</v>
       </c>
       <c r="N123" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="124" spans="1:14" x14ac:dyDescent="0.25">
@@ -3507,7 +3573,7 @@
         <v>78</v>
       </c>
       <c r="N124" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="125" spans="1:14" x14ac:dyDescent="0.25">
@@ -3540,7 +3606,7 @@
         <v>79</v>
       </c>
       <c r="N125" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="126" spans="1:14" x14ac:dyDescent="0.25">
@@ -3573,7 +3639,7 @@
         <v>80</v>
       </c>
       <c r="N126" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="127" spans="1:14" x14ac:dyDescent="0.25">
@@ -3608,7 +3674,7 @@
         <v>86</v>
       </c>
       <c r="N127" s="9" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="128" spans="1:14" x14ac:dyDescent="0.25">
@@ -3656,7 +3722,7 @@
       </c>
       <c r="M129" s="9"/>
       <c r="N129" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="130" spans="1:14" x14ac:dyDescent="0.25">
@@ -3672,7 +3738,7 @@
         <v>58</v>
       </c>
       <c r="F130" s="9" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="G130" s="9"/>
       <c r="H130" s="9"/>
@@ -3688,10 +3754,10 @@
         <v>39</v>
       </c>
       <c r="M130" s="10" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="N130" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="131" spans="1:14" x14ac:dyDescent="0.25">
@@ -3707,7 +3773,7 @@
         <v>58</v>
       </c>
       <c r="F131" s="9" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="G131" s="9"/>
       <c r="H131" s="9"/>
@@ -3723,10 +3789,10 @@
         <v>39</v>
       </c>
       <c r="M131" s="10" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="N131" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="132" spans="1:14" x14ac:dyDescent="0.25">
@@ -3742,7 +3808,7 @@
         <v>58</v>
       </c>
       <c r="F132" s="9" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="G132" s="9"/>
       <c r="H132" s="9"/>
@@ -3758,10 +3824,10 @@
         <v>39</v>
       </c>
       <c r="M132" s="10" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="N132" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="133" spans="1:14" x14ac:dyDescent="0.25">
@@ -3777,7 +3843,7 @@
         <v>58</v>
       </c>
       <c r="F133" s="9" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="G133" s="9"/>
       <c r="H133" s="9"/>
@@ -3793,12 +3859,12 @@
       </c>
       <c r="M133" s="9"/>
       <c r="N133" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="134" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B134" s="9"/>
       <c r="C134" s="9"/>
@@ -3823,12 +3889,12 @@
       </c>
       <c r="M134" s="9"/>
       <c r="N134" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="135" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B135" s="9"/>
       <c r="C135" s="9"/>
@@ -3839,7 +3905,7 @@
         <v>58</v>
       </c>
       <c r="F135" s="10" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="G135" s="9"/>
       <c r="H135" s="9"/>
@@ -3855,13 +3921,15 @@
         <v>39</v>
       </c>
       <c r="M135" s="10" t="s">
-        <v>106</v>
-      </c>
-      <c r="N135" s="9"/>
+        <v>104</v>
+      </c>
+      <c r="N135" s="9" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="136" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B136" s="9"/>
       <c r="C136" s="9"/>
@@ -3872,7 +3940,7 @@
         <v>58</v>
       </c>
       <c r="F136" s="9" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="G136" s="9"/>
       <c r="H136" s="9"/>
@@ -3888,13 +3956,15 @@
         <v>39</v>
       </c>
       <c r="M136" s="10" t="s">
-        <v>106</v>
-      </c>
-      <c r="N136" s="9"/>
+        <v>104</v>
+      </c>
+      <c r="N136" s="9" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="137" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B137" s="9"/>
       <c r="C137" s="9"/>
@@ -3905,7 +3975,7 @@
         <v>58</v>
       </c>
       <c r="F137" s="10" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
       <c r="G137" s="9"/>
       <c r="H137" s="9"/>
@@ -3921,13 +3991,15 @@
         <v>39</v>
       </c>
       <c r="M137" s="10" t="s">
-        <v>106</v>
-      </c>
-      <c r="N137" s="9"/>
+        <v>104</v>
+      </c>
+      <c r="N137" s="9" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="138" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B138" s="9"/>
       <c r="C138" s="9"/>
@@ -3938,7 +4010,7 @@
         <v>58</v>
       </c>
       <c r="F138" s="9" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="G138" s="9"/>
       <c r="H138" s="9"/>
@@ -3953,7 +4025,9 @@
         <v>39</v>
       </c>
       <c r="M138" s="9"/>
-      <c r="N138" s="9"/>
+      <c r="N138" s="9" t="s">
+        <v>99</v>
+      </c>
     </row>
     <row r="139" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A139" s="5" t="s">
@@ -3975,10 +4049,10 @@
     </row>
     <row r="140" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="C140" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="H140" t="s">
         <v>47</v>
@@ -3987,27 +4061,25 @@
         <v>88</v>
       </c>
       <c r="K140" s="22">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="L140" t="s">
         <v>39</v>
       </c>
-      <c r="M140" s="12" t="s">
-        <v>152</v>
-      </c>
+      <c r="M140" s="12"/>
       <c r="N140" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="141" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="C141" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="F141" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="H141" t="s">
         <v>47</v>
@@ -4022,15 +4094,15 @@
         <v>39</v>
       </c>
       <c r="N141" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="142" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="C142" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="H142" t="s">
         <v>45</v>
@@ -4045,19 +4117,19 @@
         <v>39</v>
       </c>
       <c r="M142" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="N142" s="9"/>
     </row>
     <row r="143" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
+        <v>142</v>
+      </c>
+      <c r="C143" t="s">
+        <v>144</v>
+      </c>
+      <c r="F143" t="s">
         <v>146</v>
-      </c>
-      <c r="C143" t="s">
-        <v>148</v>
-      </c>
-      <c r="F143" t="s">
-        <v>150</v>
       </c>
       <c r="H143" t="s">
         <v>45</v>
@@ -4093,7 +4165,7 @@
     </row>
     <row r="145" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B145" s="11"/>
       <c r="C145" s="9" t="s">
@@ -4117,12 +4189,12 @@
       </c>
       <c r="M145" s="9"/>
       <c r="N145" s="9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
     </row>
     <row r="146" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B146" s="11"/>
       <c r="C146" s="9" t="s">
@@ -4131,7 +4203,7 @@
       <c r="D146" s="11"/>
       <c r="E146" s="11"/>
       <c r="F146" s="20" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="G146" s="11"/>
       <c r="H146" s="11"/>
@@ -4147,101 +4219,105 @@
         <v>39</v>
       </c>
       <c r="M146" s="9" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="N146" s="9" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
     </row>
     <row r="147" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A147" s="11"/>
       <c r="B147" s="11"/>
-      <c r="C147" s="11"/>
+      <c r="C147" s="9"/>
       <c r="D147" s="11"/>
       <c r="E147" s="11"/>
-      <c r="F147" s="11"/>
+      <c r="F147" s="11" t="s">
+        <v>193</v>
+      </c>
       <c r="G147" s="11"/>
       <c r="H147" s="11"/>
       <c r="I147" s="11"/>
-      <c r="J147" s="11"/>
-      <c r="K147" s="11"/>
-      <c r="L147" s="9"/>
-      <c r="M147" s="9"/>
+      <c r="K147" s="21"/>
+      <c r="L147" s="10"/>
+      <c r="M147" s="11" t="s">
+        <v>194</v>
+      </c>
       <c r="N147" s="9"/>
     </row>
     <row r="148" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A148" s="3" t="s">
+      <c r="A148" s="11"/>
+      <c r="B148" s="11"/>
+      <c r="C148" s="11"/>
+      <c r="D148" s="11"/>
+      <c r="E148" s="11"/>
+      <c r="F148" s="11"/>
+      <c r="G148" s="11"/>
+      <c r="H148" s="11"/>
+      <c r="I148" s="11"/>
+      <c r="J148" s="11"/>
+      <c r="K148" s="11"/>
+      <c r="L148" s="9"/>
+      <c r="M148" s="9"/>
+      <c r="N148" s="9"/>
+    </row>
+    <row r="149" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A149" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B148" s="3"/>
-      <c r="C148" s="3"/>
-      <c r="D148" s="3"/>
-      <c r="E148" s="3"/>
-      <c r="F148" s="3"/>
-      <c r="G148" s="3"/>
-      <c r="H148" s="3"/>
-      <c r="I148" s="3"/>
-      <c r="J148" s="4"/>
-      <c r="K148" s="4"/>
-      <c r="L148" s="4"/>
-      <c r="M148" s="4"/>
-      <c r="N148" s="4"/>
-    </row>
-    <row r="149" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="J149" s="8" t="s">
+      <c r="B149" s="3"/>
+      <c r="C149" s="3"/>
+      <c r="D149" s="3"/>
+      <c r="E149" s="3"/>
+      <c r="F149" s="3"/>
+      <c r="G149" s="3"/>
+      <c r="H149" s="3"/>
+      <c r="I149" s="3"/>
+      <c r="J149" s="4"/>
+      <c r="K149" s="4"/>
+      <c r="L149" s="4"/>
+      <c r="M149" s="4"/>
+      <c r="N149" s="4"/>
+    </row>
+    <row r="150" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="J150" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="K149" s="8">
+      <c r="K150" s="8">
         <v>100</v>
       </c>
-      <c r="L149" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="M149" s="8" t="s">
+      <c r="L150" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="M150" s="8" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="150" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A150" s="5" t="s">
+    <row r="151" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A151" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B150" s="5"/>
-      <c r="C150" s="5"/>
-      <c r="D150" s="5"/>
-      <c r="E150" s="5"/>
-      <c r="F150" s="5"/>
-      <c r="G150" s="5"/>
-      <c r="H150" s="5"/>
-      <c r="I150" s="5"/>
-      <c r="J150" s="6"/>
-      <c r="K150" s="6"/>
-      <c r="L150" s="6"/>
-      <c r="M150" s="6"/>
-      <c r="N150" s="6"/>
-    </row>
-    <row r="151" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A151" t="s">
-        <v>35</v>
-      </c>
-      <c r="J151" t="s">
-        <v>41</v>
-      </c>
-      <c r="K151">
-        <v>22</v>
-      </c>
-      <c r="L151" t="s">
-        <v>39</v>
-      </c>
+      <c r="B151" s="5"/>
+      <c r="C151" s="5"/>
+      <c r="D151" s="5"/>
+      <c r="E151" s="5"/>
+      <c r="F151" s="5"/>
+      <c r="G151" s="5"/>
+      <c r="H151" s="5"/>
+      <c r="I151" s="5"/>
+      <c r="J151" s="6"/>
+      <c r="K151" s="6"/>
+      <c r="L151" s="6"/>
+      <c r="M151" s="6"/>
+      <c r="N151" s="6"/>
     </row>
     <row r="152" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="J152" t="s">
         <v>41</v>
       </c>
       <c r="K152">
-        <v>100</v>
+        <v>22</v>
       </c>
       <c r="L152" t="s">
         <v>39</v>
@@ -4249,13 +4325,13 @@
     </row>
     <row r="153" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="J153" t="s">
         <v>41</v>
       </c>
       <c r="K153">
-        <v>4</v>
+        <v>100</v>
       </c>
       <c r="L153" t="s">
         <v>39</v>
@@ -4263,13 +4339,13 @@
     </row>
     <row r="154" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>96</v>
+        <v>50</v>
       </c>
       <c r="J154" t="s">
         <v>41</v>
       </c>
       <c r="K154">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="L154" t="s">
         <v>39</v>
@@ -4283,7 +4359,7 @@
         <v>41</v>
       </c>
       <c r="K155">
-        <v>8</v>
+        <v>100</v>
       </c>
       <c r="L155" t="s">
         <v>39</v>
@@ -4297,7 +4373,7 @@
         <v>41</v>
       </c>
       <c r="K156">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="L156" t="s">
         <v>39</v>
@@ -4310,51 +4386,51 @@
       <c r="J157" t="s">
         <v>41</v>
       </c>
-      <c r="K157" s="7">
+      <c r="K157">
+        <v>1</v>
+      </c>
+      <c r="L157" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="158" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A158" t="s">
+        <v>92</v>
+      </c>
+      <c r="J158" t="s">
+        <v>41</v>
+      </c>
+      <c r="K158" s="7">
         <v>22</v>
       </c>
-      <c r="L157" s="18" t="s">
-        <v>39</v>
-      </c>
-      <c r="M157" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="158" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A158" s="5" t="s">
+      <c r="L158" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="M158" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="159" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A159" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B158" s="5"/>
-      <c r="C158" s="5"/>
-      <c r="D158" s="5"/>
-      <c r="E158" s="5"/>
-      <c r="F158" s="5"/>
-      <c r="G158" s="5"/>
-      <c r="H158" s="5"/>
-      <c r="I158" s="5"/>
-      <c r="J158" s="6"/>
-      <c r="K158" s="6"/>
-      <c r="L158" s="6"/>
-      <c r="M158" s="6"/>
-      <c r="N158" s="6"/>
-    </row>
-    <row r="159" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A159" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="J159" t="s">
-        <v>41</v>
-      </c>
-      <c r="K159" s="18">
-        <v>16</v>
-      </c>
-      <c r="L159" s="18" t="s">
-        <v>39</v>
-      </c>
+      <c r="B159" s="5"/>
+      <c r="C159" s="5"/>
+      <c r="D159" s="5"/>
+      <c r="E159" s="5"/>
+      <c r="F159" s="5"/>
+      <c r="G159" s="5"/>
+      <c r="H159" s="5"/>
+      <c r="I159" s="5"/>
+      <c r="J159" s="6"/>
+      <c r="K159" s="6"/>
+      <c r="L159" s="6"/>
+      <c r="M159" s="6"/>
+      <c r="N159" s="6"/>
     </row>
     <row r="160" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A160" s="7" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="J160" t="s">
         <v>41</v>
@@ -4368,7 +4444,7 @@
     </row>
     <row r="161" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A161" s="7" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="J161" t="s">
         <v>41</v>
@@ -4382,7 +4458,7 @@
     </row>
     <row r="162" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A162" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J162" t="s">
         <v>41</v>
@@ -4395,46 +4471,46 @@
       </c>
     </row>
     <row r="163" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A163" s="5" t="s">
+      <c r="A163" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="J163" t="s">
+        <v>41</v>
+      </c>
+      <c r="K163" s="18">
+        <v>16</v>
+      </c>
+      <c r="L163" s="18" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="164" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A164" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B163" s="5"/>
-      <c r="C163" s="5"/>
-      <c r="D163" s="5"/>
-      <c r="E163" s="5"/>
-      <c r="F163" s="5"/>
-      <c r="G163" s="5"/>
-      <c r="H163" s="5"/>
-      <c r="I163" s="5"/>
-      <c r="J163" s="6"/>
-      <c r="K163" s="6"/>
-      <c r="L163" s="6"/>
-      <c r="M163" s="6"/>
-      <c r="N163" s="6"/>
-    </row>
-    <row r="164" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A164" s="18" t="s">
-        <v>157</v>
-      </c>
-      <c r="J164" t="s">
-        <v>41</v>
-      </c>
-      <c r="K164">
-        <v>7</v>
-      </c>
-      <c r="L164" s="18" t="s">
-        <v>39</v>
-      </c>
+      <c r="B164" s="5"/>
+      <c r="C164" s="5"/>
+      <c r="D164" s="5"/>
+      <c r="E164" s="5"/>
+      <c r="F164" s="5"/>
+      <c r="G164" s="5"/>
+      <c r="H164" s="5"/>
+      <c r="I164" s="5"/>
+      <c r="J164" s="6"/>
+      <c r="K164" s="6"/>
+      <c r="L164" s="6"/>
+      <c r="M164" s="6"/>
+      <c r="N164" s="6"/>
     </row>
     <row r="165" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A165" s="18" t="s">
-        <v>163</v>
+        <v>151</v>
       </c>
       <c r="J165" t="s">
         <v>41</v>
       </c>
-      <c r="K165" s="18">
-        <v>35</v>
+      <c r="K165">
+        <v>7</v>
       </c>
       <c r="L165" s="18" t="s">
         <v>39</v>
@@ -4442,13 +4518,13 @@
     </row>
     <row r="166" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A166" s="18" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="J166" t="s">
         <v>41</v>
       </c>
       <c r="K166" s="18">
-        <v>63</v>
+        <v>35</v>
       </c>
       <c r="L166" s="18" t="s">
         <v>39</v>
@@ -4456,61 +4532,59 @@
     </row>
     <row r="167" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A167" s="18" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="J167" t="s">
         <v>41</v>
       </c>
-      <c r="K167" s="7">
-        <v>40</v>
+      <c r="K167" s="18">
+        <v>63</v>
       </c>
       <c r="L167" s="18" t="s">
         <v>39</v>
-      </c>
-      <c r="M167" s="7" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="168" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A168" s="18" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="J168" t="s">
         <v>41</v>
       </c>
-      <c r="K168" s="7">
-        <v>70</v>
+      <c r="K168" s="18">
+        <v>54</v>
       </c>
       <c r="L168" s="18" t="s">
         <v>39</v>
       </c>
-      <c r="M168" s="7" t="s">
-        <v>173</v>
-      </c>
+      <c r="M168" s="7"/>
     </row>
     <row r="169" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A169" s="18" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="J169" t="s">
         <v>41</v>
       </c>
-      <c r="K169" s="18">
-        <v>10</v>
+      <c r="K169" s="7">
+        <v>70</v>
       </c>
       <c r="L169" s="18" t="s">
         <v>39</v>
+      </c>
+      <c r="M169" s="7" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="170" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A170" s="18" t="s">
-        <v>120</v>
+        <v>156</v>
       </c>
       <c r="J170" t="s">
         <v>41</v>
       </c>
       <c r="K170" s="18">
-        <v>90</v>
+        <v>10</v>
       </c>
       <c r="L170" s="18" t="s">
         <v>39</v>
@@ -4518,13 +4592,13 @@
     </row>
     <row r="171" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A171" s="18" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="J171" t="s">
         <v>41</v>
       </c>
       <c r="K171" s="18">
-        <v>46</v>
+        <v>90</v>
       </c>
       <c r="L171" s="18" t="s">
         <v>39</v>
@@ -4532,119 +4606,119 @@
     </row>
     <row r="172" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A172" s="18" t="s">
-        <v>170</v>
+        <v>119</v>
       </c>
       <c r="J172" t="s">
         <v>41</v>
       </c>
-      <c r="K172" s="7">
+      <c r="K172" s="18">
+        <v>46</v>
+      </c>
+      <c r="L172" s="18" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="173" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A173" s="18" t="s">
+        <v>164</v>
+      </c>
+      <c r="J173" t="s">
+        <v>41</v>
+      </c>
+      <c r="K173" s="7">
         <v>0</v>
       </c>
-      <c r="L172" s="18" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="173" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A173" s="5" t="s">
+      <c r="L173" s="18" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="174" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A174" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="B173" s="5"/>
-      <c r="C173" s="5"/>
-      <c r="D173" s="5"/>
-      <c r="E173" s="5"/>
-      <c r="F173" s="5"/>
-      <c r="G173" s="5"/>
-      <c r="H173" s="5"/>
-      <c r="I173" s="5"/>
-      <c r="J173" s="6"/>
-      <c r="K173" s="6"/>
-      <c r="L173" s="6"/>
-      <c r="M173" s="6"/>
-      <c r="N173" s="6"/>
-    </row>
-    <row r="174" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A174" s="7" t="s">
+      <c r="B174" s="5"/>
+      <c r="C174" s="5"/>
+      <c r="D174" s="5"/>
+      <c r="E174" s="5"/>
+      <c r="F174" s="5"/>
+      <c r="G174" s="5"/>
+      <c r="H174" s="5"/>
+      <c r="I174" s="5"/>
+      <c r="J174" s="6"/>
+      <c r="K174" s="6"/>
+      <c r="L174" s="6"/>
+      <c r="M174" s="6"/>
+      <c r="N174" s="6"/>
+    </row>
+    <row r="175" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A175" s="7" t="s">
         <v>65</v>
       </c>
-      <c r="J174" t="s">
+      <c r="J175" t="s">
         <v>41</v>
       </c>
-      <c r="K174" s="14">
+      <c r="K175" s="14">
         <f>8.5*20/(29.5+8.5)</f>
         <v>4.4736842105263159</v>
       </c>
-      <c r="L174" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="175" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A175" s="7" t="s">
+      <c r="L175" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="176" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A176" s="7" t="s">
         <v>64</v>
       </c>
-      <c r="J175" t="s">
+      <c r="J176" t="s">
         <v>41</v>
       </c>
-      <c r="K175" s="14">
+      <c r="K176" s="14">
         <f>(80.7*0+14.4*20+0.3*5*0)/(80.7+14.4+0.3*5)</f>
         <v>2.981366459627329</v>
       </c>
-      <c r="L175" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="176" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A176" s="7" t="s">
+      <c r="L176" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="177" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A177" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="J176" t="s">
+      <c r="J177" t="s">
         <v>41</v>
       </c>
-      <c r="K176" s="14">
+      <c r="K177" s="14">
         <f>(45.6*0+44.1*20+1.3*5*0+1.8*10*0)/(45.6+44.1+1.3*5+1.8*10)</f>
         <v>7.723292469352014</v>
       </c>
-      <c r="L176" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="177" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A177" s="7" t="s">
+      <c r="L177" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="178" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A178" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="J177" t="s">
+      <c r="J178" t="s">
         <v>41</v>
       </c>
-      <c r="K177">
+      <c r="K178">
         <f>60</f>
         <v>60</v>
       </c>
-      <c r="L177" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="178" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A178" s="7" t="s">
-        <v>71</v>
-      </c>
-      <c r="J178" t="s">
-        <v>41</v>
-      </c>
-      <c r="K178">
-        <v>0</v>
-      </c>
       <c r="L178" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="179" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A179" s="7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="J179" t="s">
         <v>41</v>
       </c>
       <c r="K179">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="L179" t="s">
         <v>39</v>
@@ -4652,7 +4726,7 @@
     </row>
     <row r="180" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A180" s="7" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="J180" t="s">
         <v>41</v>
@@ -4666,7 +4740,7 @@
     </row>
     <row r="181" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A181" s="7" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="J181" t="s">
         <v>41</v>
@@ -4680,236 +4754,227 @@
     </row>
     <row r="182" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A182" s="7" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="J182" t="s">
         <v>41</v>
       </c>
       <c r="K182">
+        <v>20</v>
+      </c>
+      <c r="L182" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="183" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A183" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="J183" t="s">
+        <v>41</v>
+      </c>
+      <c r="K183">
         <f>43</f>
         <v>43</v>
       </c>
-      <c r="L182" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="183" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A183" s="5" t="s">
+      <c r="L183" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="184" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A184" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B183" s="5"/>
-      <c r="C183" s="5"/>
-      <c r="D183" s="5"/>
-      <c r="E183" s="5"/>
-      <c r="F183" s="5"/>
-      <c r="G183" s="5"/>
-      <c r="H183" s="5"/>
-      <c r="I183" s="5"/>
-      <c r="J183" s="6"/>
-      <c r="K183" s="6"/>
-      <c r="L183" s="6"/>
-      <c r="M183" s="6"/>
-      <c r="N183" s="6"/>
-    </row>
-    <row r="184" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A184" t="s">
-        <v>57</v>
-      </c>
-      <c r="J184" t="s">
-        <v>41</v>
-      </c>
-      <c r="K184">
-        <v>36</v>
-      </c>
-      <c r="L184" t="s">
-        <v>39</v>
-      </c>
+      <c r="B184" s="5"/>
+      <c r="C184" s="5"/>
+      <c r="D184" s="5"/>
+      <c r="E184" s="5"/>
+      <c r="F184" s="5"/>
+      <c r="G184" s="5"/>
+      <c r="H184" s="5"/>
+      <c r="I184" s="5"/>
+      <c r="J184" s="6"/>
+      <c r="K184" s="6"/>
+      <c r="L184" s="6"/>
+      <c r="M184" s="6"/>
+      <c r="N184" s="6"/>
     </row>
     <row r="185" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
-        <v>104</v>
+        <v>57</v>
       </c>
       <c r="J185" t="s">
         <v>41</v>
       </c>
-      <c r="K185" s="18">
+      <c r="K185">
+        <v>36</v>
+      </c>
+      <c r="L185" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="186" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A186" t="s">
+        <v>102</v>
+      </c>
+      <c r="J186" t="s">
+        <v>41</v>
+      </c>
+      <c r="K186" s="18">
         <v>43</v>
       </c>
-      <c r="L185" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="186" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A186" s="5" t="s">
+      <c r="L186" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="187" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A187" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B186" s="5"/>
-      <c r="C186" s="5"/>
-      <c r="D186" s="5"/>
-      <c r="E186" s="5"/>
-      <c r="F186" s="5"/>
-      <c r="G186" s="5"/>
-      <c r="H186" s="5"/>
-      <c r="I186" s="5"/>
-      <c r="J186" s="6"/>
-      <c r="K186" s="6"/>
-      <c r="L186" s="6"/>
-      <c r="M186" s="6"/>
-      <c r="N186" s="6"/>
-    </row>
-    <row r="187" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A187" t="s">
-        <v>146</v>
-      </c>
-      <c r="J187" t="s">
+      <c r="B187" s="5"/>
+      <c r="C187" s="5"/>
+      <c r="D187" s="5"/>
+      <c r="E187" s="5"/>
+      <c r="F187" s="5"/>
+      <c r="G187" s="5"/>
+      <c r="H187" s="5"/>
+      <c r="I187" s="5"/>
+      <c r="J187" s="6"/>
+      <c r="K187" s="6"/>
+      <c r="L187" s="6"/>
+      <c r="M187" s="6"/>
+      <c r="N187" s="6"/>
+    </row>
+    <row r="188" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A188" t="s">
+        <v>142</v>
+      </c>
+      <c r="J188" t="s">
         <v>41</v>
       </c>
-      <c r="K187" s="16">
+      <c r="K188" s="16">
         <v>52</v>
       </c>
-      <c r="L187" t="s">
-        <v>39</v>
-      </c>
-      <c r="M187" s="25"/>
-    </row>
-    <row r="188" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A188" s="5" t="s">
+      <c r="L188" t="s">
+        <v>39</v>
+      </c>
+      <c r="M188" s="25"/>
+    </row>
+    <row r="189" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A189" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B188" s="5"/>
-      <c r="C188" s="5"/>
-      <c r="D188" s="5"/>
-      <c r="E188" s="5"/>
-      <c r="F188" s="5"/>
-      <c r="G188" s="5"/>
-      <c r="H188" s="5"/>
-      <c r="I188" s="5"/>
-      <c r="J188" s="6"/>
-      <c r="K188" s="6"/>
-      <c r="L188" s="6"/>
-      <c r="M188" s="6"/>
-      <c r="N188" s="6"/>
-    </row>
-    <row r="189" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A189" t="s">
-        <v>125</v>
-      </c>
-      <c r="J189" t="s">
+      <c r="B189" s="5"/>
+      <c r="C189" s="5"/>
+      <c r="D189" s="5"/>
+      <c r="E189" s="5"/>
+      <c r="F189" s="5"/>
+      <c r="G189" s="5"/>
+      <c r="H189" s="5"/>
+      <c r="I189" s="5"/>
+      <c r="J189" s="6"/>
+      <c r="K189" s="6"/>
+      <c r="L189" s="6"/>
+      <c r="M189" s="6"/>
+      <c r="N189" s="6"/>
+    </row>
+    <row r="190" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A190" t="s">
+        <v>121</v>
+      </c>
+      <c r="J190" t="s">
         <v>41</v>
       </c>
-      <c r="K189">
+      <c r="K190">
         <v>4</v>
       </c>
-      <c r="L189" t="s">
-        <v>39</v>
-      </c>
-      <c r="M189" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="191" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A191" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="B191" s="3"/>
-      <c r="C191" s="3"/>
-      <c r="D191" s="3"/>
-      <c r="E191" s="3"/>
-      <c r="F191" s="3"/>
-      <c r="G191" s="3"/>
-      <c r="H191" s="3"/>
-      <c r="I191" s="3"/>
-      <c r="J191" s="4"/>
-      <c r="K191" s="4"/>
-      <c r="L191" s="4"/>
-      <c r="M191" s="4"/>
-      <c r="N191" s="4"/>
+      <c r="L190" t="s">
+        <v>39</v>
+      </c>
+      <c r="M190" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="192" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="G192" s="8"/>
-      <c r="H192" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="I192" s="8"/>
-      <c r="J192" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="K192" s="8">
-        <v>-100</v>
-      </c>
-      <c r="L192" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="M192" s="8" t="s">
-        <v>90</v>
-      </c>
+      <c r="A192" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="B192" s="3"/>
+      <c r="C192" s="3"/>
+      <c r="D192" s="3"/>
+      <c r="E192" s="3"/>
+      <c r="F192" s="3"/>
+      <c r="G192" s="3"/>
+      <c r="H192" s="3"/>
+      <c r="I192" s="3"/>
+      <c r="J192" s="4"/>
+      <c r="K192" s="4"/>
+      <c r="L192" s="4"/>
+      <c r="M192" s="4"/>
+      <c r="N192" s="4"/>
     </row>
     <row r="193" spans="1:14" x14ac:dyDescent="0.25">
       <c r="G193" s="8"/>
       <c r="H193" s="8" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="I193" s="8"/>
       <c r="J193" s="8" t="s">
         <v>42</v>
       </c>
       <c r="K193" s="8">
+        <v>-100</v>
+      </c>
+      <c r="L193" s="8" t="s">
+        <v>48</v>
+      </c>
+      <c r="M193" s="8" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="194" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="G194" s="8"/>
+      <c r="H194" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="I194" s="8"/>
+      <c r="J194" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="K194" s="8">
         <v>0</v>
       </c>
-      <c r="L193" s="8" t="s">
-        <v>39</v>
-      </c>
-      <c r="M193" s="8" t="s">
+      <c r="L194" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="M194" s="8" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="194" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A194" s="5" t="s">
+    <row r="195" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A195" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="B194" s="5"/>
-      <c r="C194" s="5"/>
-      <c r="D194" s="5"/>
-      <c r="E194" s="5"/>
-      <c r="F194" s="5"/>
-      <c r="G194" s="5"/>
-      <c r="H194" s="5"/>
-      <c r="I194" s="5"/>
-      <c r="J194" s="6"/>
-      <c r="K194" s="6"/>
-      <c r="L194" s="6"/>
-      <c r="M194" s="6"/>
-      <c r="N194" s="6"/>
-    </row>
-    <row r="195" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A195" t="s">
-        <v>35</v>
-      </c>
-      <c r="G195" t="s">
-        <v>91</v>
-      </c>
-      <c r="H195" t="s">
-        <v>45</v>
-      </c>
-      <c r="J195" t="s">
-        <v>42</v>
-      </c>
-      <c r="K195" s="18">
-        <v>5.3</v>
-      </c>
-      <c r="L195" t="s">
-        <v>39</v>
-      </c>
-      <c r="N195" t="s">
-        <v>108</v>
-      </c>
+      <c r="B195" s="5"/>
+      <c r="C195" s="5"/>
+      <c r="D195" s="5"/>
+      <c r="E195" s="5"/>
+      <c r="F195" s="5"/>
+      <c r="G195" s="5"/>
+      <c r="H195" s="5"/>
+      <c r="I195" s="5"/>
+      <c r="J195" s="6"/>
+      <c r="K195" s="6"/>
+      <c r="L195" s="6"/>
+      <c r="M195" s="6"/>
+      <c r="N195" s="6"/>
     </row>
     <row r="196" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="G196" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H196" t="s">
         <v>45</v>
@@ -4918,21 +4983,24 @@
         <v>42</v>
       </c>
       <c r="K196" s="18">
-        <v>4.9000000000000004</v>
+        <v>5.3</v>
       </c>
       <c r="L196" t="s">
         <v>39</v>
       </c>
+      <c r="M196" t="s">
+        <v>185</v>
+      </c>
       <c r="N196" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="197" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
-        <v>95</v>
+        <v>50</v>
       </c>
       <c r="G197" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H197" t="s">
         <v>45</v>
@@ -4941,13 +5009,16 @@
         <v>42</v>
       </c>
       <c r="K197" s="18">
-        <v>12.7</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="L197" t="s">
         <v>39</v>
       </c>
+      <c r="M197" t="s">
+        <v>185</v>
+      </c>
       <c r="N197" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="198" spans="1:14" x14ac:dyDescent="0.25">
@@ -4955,7 +5026,7 @@
         <v>94</v>
       </c>
       <c r="G198" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H198" t="s">
         <v>45</v>
@@ -4964,13 +5035,16 @@
         <v>42</v>
       </c>
       <c r="K198" s="18">
-        <v>15.7</v>
+        <v>12.7</v>
       </c>
       <c r="L198" t="s">
         <v>39</v>
       </c>
+      <c r="M198" t="s">
+        <v>185</v>
+      </c>
       <c r="N198" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="199" spans="1:14" x14ac:dyDescent="0.25">
@@ -4978,7 +5052,7 @@
         <v>93</v>
       </c>
       <c r="G199" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H199" t="s">
         <v>45</v>
@@ -4986,57 +5060,63 @@
       <c r="J199" t="s">
         <v>42</v>
       </c>
-      <c r="K199" s="7">
+      <c r="K199" s="18">
+        <v>24</v>
+      </c>
+      <c r="L199" t="s">
+        <v>39</v>
+      </c>
+      <c r="M199" t="s">
+        <v>186</v>
+      </c>
+      <c r="N199" s="27" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="200" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A200" t="s">
+        <v>92</v>
+      </c>
+      <c r="G200" t="s">
+        <v>90</v>
+      </c>
+      <c r="H200" t="s">
+        <v>45</v>
+      </c>
+      <c r="J200" t="s">
+        <v>42</v>
+      </c>
+      <c r="K200" s="7">
         <v>10</v>
       </c>
-      <c r="L199" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="200" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A200" s="5" t="s">
+      <c r="L200" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="201" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A201" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B200" s="5"/>
-      <c r="C200" s="5"/>
-      <c r="D200" s="5"/>
-      <c r="E200" s="5"/>
-      <c r="F200" s="5"/>
-      <c r="G200" s="5"/>
-      <c r="H200" s="5"/>
-      <c r="I200" s="5"/>
-      <c r="J200" s="6"/>
-      <c r="K200" s="6"/>
-      <c r="L200" s="6"/>
-      <c r="M200" s="6"/>
-      <c r="N200" s="6"/>
-    </row>
-    <row r="201" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A201" s="7" t="s">
-        <v>109</v>
-      </c>
-      <c r="G201" t="s">
-        <v>91</v>
-      </c>
-      <c r="H201" t="s">
-        <v>45</v>
-      </c>
-      <c r="J201" t="s">
-        <v>42</v>
-      </c>
-      <c r="K201" s="7">
-        <v>5</v>
-      </c>
-      <c r="L201" t="s">
-        <v>39</v>
-      </c>
+      <c r="B201" s="5"/>
+      <c r="C201" s="5"/>
+      <c r="D201" s="5"/>
+      <c r="E201" s="5"/>
+      <c r="F201" s="5"/>
+      <c r="G201" s="5"/>
+      <c r="H201" s="5"/>
+      <c r="I201" s="5"/>
+      <c r="J201" s="6"/>
+      <c r="K201" s="6"/>
+      <c r="L201" s="6"/>
+      <c r="M201" s="6"/>
+      <c r="N201" s="6"/>
     </row>
     <row r="202" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A202" s="7" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="G202" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H202" t="s">
         <v>45</v>
@@ -5044,19 +5124,22 @@
       <c r="J202" t="s">
         <v>42</v>
       </c>
-      <c r="K202" s="7">
-        <v>5</v>
+      <c r="K202" s="18">
+        <v>12</v>
       </c>
       <c r="L202" t="s">
         <v>39</v>
+      </c>
+      <c r="N202" s="27" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="203" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A203" s="7" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="G203" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H203" t="s">
         <v>45</v>
@@ -5064,19 +5147,22 @@
       <c r="J203" t="s">
         <v>42</v>
       </c>
-      <c r="K203" s="7">
-        <v>5</v>
+      <c r="K203" s="18">
+        <v>12</v>
       </c>
       <c r="L203" t="s">
         <v>39</v>
+      </c>
+      <c r="N203" s="27" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="204" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A204" s="7" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G204" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H204" t="s">
         <v>45</v>
@@ -5084,57 +5170,57 @@
       <c r="J204" t="s">
         <v>42</v>
       </c>
-      <c r="K204" s="7">
-        <v>5</v>
+      <c r="K204" s="18">
+        <v>0</v>
       </c>
       <c r="L204" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="205" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A205" s="5" t="s">
+      <c r="A205" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="G205" t="s">
+        <v>90</v>
+      </c>
+      <c r="H205" t="s">
+        <v>45</v>
+      </c>
+      <c r="J205" t="s">
+        <v>42</v>
+      </c>
+      <c r="K205" s="18">
+        <v>0</v>
+      </c>
+      <c r="L205" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="206" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A206" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B205" s="5"/>
-      <c r="C205" s="5"/>
-      <c r="D205" s="5"/>
-      <c r="E205" s="5"/>
-      <c r="F205" s="5"/>
-      <c r="G205" s="5"/>
-      <c r="H205" s="5"/>
-      <c r="I205" s="5"/>
-      <c r="J205" s="6"/>
-      <c r="K205" s="6"/>
-      <c r="L205" s="6"/>
-      <c r="M205" s="6"/>
-      <c r="N205" s="6"/>
-    </row>
-    <row r="206" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A206" s="18" t="s">
-        <v>120</v>
-      </c>
-      <c r="G206" t="s">
-        <v>91</v>
-      </c>
-      <c r="H206" t="s">
-        <v>45</v>
-      </c>
-      <c r="J206" t="s">
-        <v>42</v>
-      </c>
-      <c r="K206" s="7">
-        <v>1</v>
-      </c>
-      <c r="L206" t="s">
-        <v>39</v>
-      </c>
+      <c r="B206" s="5"/>
+      <c r="C206" s="5"/>
+      <c r="D206" s="5"/>
+      <c r="E206" s="5"/>
+      <c r="F206" s="5"/>
+      <c r="G206" s="5"/>
+      <c r="H206" s="5"/>
+      <c r="I206" s="5"/>
+      <c r="J206" s="6"/>
+      <c r="K206" s="6"/>
+      <c r="L206" s="6"/>
+      <c r="M206" s="6"/>
+      <c r="N206" s="6"/>
     </row>
     <row r="207" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A207" s="18" t="s">
-        <v>123</v>
+        <v>151</v>
       </c>
       <c r="G207" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H207" t="s">
         <v>45</v>
@@ -5142,82 +5228,82 @@
       <c r="J207" t="s">
         <v>42</v>
       </c>
-      <c r="K207" s="7">
-        <v>1</v>
+      <c r="K207" s="18">
+        <v>25</v>
       </c>
       <c r="L207" t="s">
         <v>39</v>
       </c>
+      <c r="M207" t="s">
+        <v>188</v>
+      </c>
+      <c r="N207" s="27" t="s">
+        <v>183</v>
+      </c>
     </row>
     <row r="208" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A208" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="B208" s="5"/>
-      <c r="C208" s="5"/>
-      <c r="D208" s="5"/>
-      <c r="E208" s="5"/>
-      <c r="F208" s="5"/>
-      <c r="G208" s="5"/>
-      <c r="H208" s="5"/>
-      <c r="I208" s="5"/>
-      <c r="J208" s="6"/>
-      <c r="K208" s="6"/>
-      <c r="L208" s="6"/>
-      <c r="M208" s="6"/>
-      <c r="N208" s="6"/>
+      <c r="A208" s="18" t="s">
+        <v>157</v>
+      </c>
+      <c r="G208" t="s">
+        <v>90</v>
+      </c>
+      <c r="H208" t="s">
+        <v>45</v>
+      </c>
+      <c r="J208" t="s">
+        <v>42</v>
+      </c>
+      <c r="K208" s="18">
+        <v>13</v>
+      </c>
+      <c r="L208" t="s">
+        <v>39</v>
+      </c>
+      <c r="M208" t="s">
+        <v>189</v>
+      </c>
+      <c r="N208" s="27" t="s">
+        <v>183</v>
+      </c>
     </row>
     <row r="209" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A209" s="7"/>
-      <c r="B209" t="s">
-        <v>84</v>
-      </c>
-      <c r="G209" t="s">
-        <v>91</v>
-      </c>
-      <c r="H209" t="s">
+      <c r="A209" s="18"/>
+      <c r="K209" s="18"/>
+      <c r="N209" s="27"/>
+    </row>
+    <row r="210" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A210" s="18" t="s">
+        <v>154</v>
+      </c>
+      <c r="G210" t="s">
+        <v>90</v>
+      </c>
+      <c r="H210" t="s">
         <v>45</v>
       </c>
-      <c r="J209" t="s">
+      <c r="J210" t="s">
         <v>42</v>
       </c>
-      <c r="K209" s="16">
-        <v>17</v>
-      </c>
-      <c r="L209" t="s">
-        <v>39</v>
-      </c>
-      <c r="M209" t="s">
-        <v>103</v>
-      </c>
-      <c r="N209" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="210" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A210" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="B210" s="5"/>
-      <c r="C210" s="5"/>
-      <c r="D210" s="5"/>
-      <c r="E210" s="5"/>
-      <c r="F210" s="5"/>
-      <c r="G210" s="5"/>
-      <c r="H210" s="5"/>
-      <c r="I210" s="5"/>
-      <c r="J210" s="6"/>
-      <c r="K210" s="6"/>
-      <c r="L210" s="6"/>
-      <c r="M210" s="6"/>
-      <c r="N210" s="6"/>
+      <c r="K210" s="18">
+        <v>19</v>
+      </c>
+      <c r="L210" t="s">
+        <v>39</v>
+      </c>
+      <c r="M210" t="s">
+        <v>187</v>
+      </c>
+      <c r="N210" s="27" t="s">
+        <v>183</v>
+      </c>
     </row>
     <row r="211" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A211" t="s">
-        <v>57</v>
+      <c r="A211" s="18" t="s">
+        <v>116</v>
       </c>
       <c r="G211" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H211" t="s">
         <v>45</v>
@@ -5225,19 +5311,25 @@
       <c r="J211" t="s">
         <v>42</v>
       </c>
-      <c r="K211" s="7">
-        <v>2.4</v>
+      <c r="K211" s="18">
+        <v>9</v>
       </c>
       <c r="L211" t="s">
         <v>39</v>
       </c>
+      <c r="M211" t="s">
+        <v>191</v>
+      </c>
+      <c r="N211" s="27" t="s">
+        <v>183</v>
+      </c>
     </row>
     <row r="212" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A212" t="s">
-        <v>104</v>
+      <c r="A212" s="18" t="s">
+        <v>119</v>
       </c>
       <c r="G212" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H212" t="s">
         <v>45</v>
@@ -5245,16 +5337,22 @@
       <c r="J212" t="s">
         <v>42</v>
       </c>
-      <c r="K212">
-        <v>15.4</v>
+      <c r="K212" s="18">
+        <v>11</v>
       </c>
       <c r="L212" t="s">
         <v>39</v>
+      </c>
+      <c r="M212" s="27" t="s">
+        <v>190</v>
+      </c>
+      <c r="N212" s="27" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="213" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A213" s="5" t="s">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="B213" s="5"/>
       <c r="C213" s="5"/>
@@ -5271,11 +5369,12 @@
       <c r="N213" s="6"/>
     </row>
     <row r="214" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A214" t="s">
-        <v>146</v>
+      <c r="A214" s="7"/>
+      <c r="B214" t="s">
+        <v>84</v>
       </c>
       <c r="G214" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H214" t="s">
         <v>45</v>
@@ -5283,16 +5382,22 @@
       <c r="J214" t="s">
         <v>42</v>
       </c>
-      <c r="K214" s="24">
-        <v>1</v>
+      <c r="K214" s="16">
+        <v>17</v>
       </c>
       <c r="L214" t="s">
         <v>39</v>
+      </c>
+      <c r="M214" t="s">
+        <v>184</v>
+      </c>
+      <c r="N214" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="215" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A215" s="5" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="B215" s="5"/>
       <c r="C215" s="5"/>
@@ -5310,10 +5415,10 @@
     </row>
     <row r="216" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>125</v>
+        <v>57</v>
       </c>
       <c r="G216" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="H216" t="s">
         <v>45</v>
@@ -5321,14 +5426,194 @@
       <c r="J216" t="s">
         <v>42</v>
       </c>
-      <c r="K216" s="18">
-        <v>4.9000000000000004</v>
+      <c r="K216" s="7">
+        <v>2.4</v>
       </c>
       <c r="L216" t="s">
         <v>39</v>
       </c>
-      <c r="M216" t="s">
-        <v>127</v>
+    </row>
+    <row r="217" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A217" t="s">
+        <v>102</v>
+      </c>
+      <c r="G217" t="s">
+        <v>90</v>
+      </c>
+      <c r="H217" t="s">
+        <v>45</v>
+      </c>
+      <c r="J217" t="s">
+        <v>42</v>
+      </c>
+      <c r="K217" s="7">
+        <v>15.4</v>
+      </c>
+      <c r="L217" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="218" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A218" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B218" s="5"/>
+      <c r="C218" s="5"/>
+      <c r="D218" s="5"/>
+      <c r="E218" s="5"/>
+      <c r="F218" s="5"/>
+      <c r="G218" s="5"/>
+      <c r="H218" s="5"/>
+      <c r="I218" s="5"/>
+      <c r="J218" s="6"/>
+      <c r="K218" s="6"/>
+      <c r="L218" s="6"/>
+      <c r="M218" s="6"/>
+      <c r="N218" s="6"/>
+    </row>
+    <row r="219" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A219" t="s">
+        <v>142</v>
+      </c>
+      <c r="G219" t="s">
+        <v>90</v>
+      </c>
+      <c r="H219" t="s">
+        <v>45</v>
+      </c>
+      <c r="J219" t="s">
+        <v>42</v>
+      </c>
+      <c r="K219" s="24">
+        <v>1</v>
+      </c>
+      <c r="L219" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="220" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A220" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="B220" s="5"/>
+      <c r="C220" s="5"/>
+      <c r="D220" s="5"/>
+      <c r="E220" s="5"/>
+      <c r="F220" s="5"/>
+      <c r="G220" s="5"/>
+      <c r="H220" s="5"/>
+      <c r="I220" s="5"/>
+      <c r="J220" s="6"/>
+      <c r="K220" s="6"/>
+      <c r="L220" s="6"/>
+      <c r="M220" s="6"/>
+      <c r="N220" s="6"/>
+    </row>
+    <row r="221" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A221" t="s">
+        <v>121</v>
+      </c>
+      <c r="G221" t="s">
+        <v>90</v>
+      </c>
+      <c r="H221" t="s">
+        <v>45</v>
+      </c>
+      <c r="J221" t="s">
+        <v>42</v>
+      </c>
+      <c r="K221" s="18">
+        <v>8</v>
+      </c>
+      <c r="L221" t="s">
+        <v>39</v>
+      </c>
+      <c r="M221" t="s">
+        <v>182</v>
+      </c>
+      <c r="N221" s="27" t="s">
+        <v>183</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="E8:E24"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="8" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E8" s="26" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="9" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E9" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="10" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E10" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="11" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E11" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="12" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E12" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="13" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E13" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="15" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E15" s="26" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="16" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E16" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="17" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E17" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="19" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E19" s="26" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="20" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E20" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="21" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E21" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="23" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E23" s="26" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="24" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="E24" t="s">
+        <v>181</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Name fix for sugar by-products
</commit_message>
<xml_diff>
--- a/data/prod_parameters/Diet.xlsx
+++ b/data/prod_parameters/Diet.xlsx
@@ -797,10 +797,10 @@
     </r>
   </si>
   <si>
-    <t>beet pulp</t>
-  </si>
-  <si>
-    <t>molasses</t>
+    <t>sugar beet pulp</t>
+  </si>
+  <si>
+    <t>sugar beet molasses</t>
   </si>
 </sst>
 </file>

</xml_diff>